<commit_message>
Update topic news feed (weekly)
</commit_message>
<xml_diff>
--- a/data/weekly/topic_feeds_2026-W06.xlsx
+++ b/data/weekly/topic_feeds_2026-W06.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -602,24 +602,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Global Report Highlights Policy Gaps in Hepatitis Elimination Efforts - European Medical Journal</t>
+          <t>ETS Nigeria Conflict Situation Report #109: January 2026 - ReliefWeb</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 10:05:57 GMT</t>
+          <t>Mon, 02 Feb 2026 09:33:09 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNTFdtYWFiNUxhMzdOMTRvYjQ3X1ZpSUpydnJ6NlpHdXhZbURWdE85WnhwX1VBd3JsVDVkQ20wbGdheHF1Umkza0syLVotaEVDSEJKYjZfSnpZREtzTjZ4d2Y3cnpqWk1EZ25iTWFDem5mN3dFX2czM2dta2NvNW5qVDNLMFRYQ2ZWS0ZSeENSNFlmRVRfbzZ6T2FSTllpejVpanNqRkdKOXJLcy1fTUxSWkZRYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOY2RLR1BHd1ZqN1d2c05HS0luYXYyUTB2ZGVhaFp6WFhmVW1yekJtY29oakx1OXc4VjA4bjVNUVdMX09YSldURkVOTjdPaWlmZE02S0xpWVVQVlRHUDZXd0VoYXZtZTFoU0V0VHV1SXBIRnM4aV94UUd2VkdOMGJfTGFBTV9pdDRWMldEcW5HNDl6UXV3b0E?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>7</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46052.42079861111</v>
+        <v>46055.39802083333</v>
       </c>
     </row>
     <row r="7">
@@ -800,24 +800,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>UK manufacturers recalibrate trade strategies as tariffs bite - Relocate magazine</t>
+          <t>Logistics Manager Magazine February 2026 - Logistics Manager</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:43:42 GMT</t>
+          <t>Mon, 02 Feb 2026 12:00:25 GMT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNVhoOENKNGhOeVEtZTU1RlB5ZVZ3Zm1Obkw3Xzg3MVFXUnFkZ1ozZmJKZUZKSGhyNmNtMGZfTjRsOHFkLUxUTWMyUzRBbGx3RTRFZU5DQ1ZCODdZSXRTa0V6WmdyeUVqSHA4amw2NEtHNXNmVG1wdEFqOWRPSWlDei1Zcm10a1BvbzQwUi1kb3F6ZWdZeFNXbmV4RS1Gcm9YSkpmUmZBcUw4QnM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5WM3c1Um9FY0RtamoxcENreVJvWUpQbWl0ODFqb0VUX0tqTk8xTVM4SmRkc21FLWJJV3pnNVhUcDlUbU5CRHpNWGhNcjRidTVHZ0Qxd09zaWFZV3NIc01mWlpYQ1ZVZ2dYTUtiMEt5ZGRCWVc3dTl2c1pNZ3ozVEE?oc=5</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>7</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46055.44701388889</v>
+        <v>46055.50028935185</v>
       </c>
     </row>
     <row r="13">
@@ -833,24 +833,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Price of consumer goods could surge as shipping costs soar, industry body says - The Guardian</t>
+          <t>UK manufacturers recalibrate trade strategies as tariffs bite - Relocate magazine</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 13:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 10:43:42 GMT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNM2ZMdGRNWlRFaVVqVHg2Q0Q3X0c1Um5uRFEzRnJselR5czM5OXJZdHdCOVpnUGxtbXo3VUlTekowNkZMaEgyeEtBeDVDUEZfSXhyZG80NlQ4bFp1cnFwTVdCdURyRnk5Zzc0N2doM1BqSFBIY25Jb2dMdUhCclVTZV93XzNsQm9VN1R3VFY3ejB6eVQ4M1ZGRmI4SV9FdEhCcXI0VEdIQVAzVjV6bHBDdmNwZzlzd2c5OVpuNmVaa09vWmdFcjBKQkJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNVhoOENKNGhOeVEtZTU1RlB5ZVZ3Zm1Obkw3Xzg3MVFXUnFkZ1ozZmJKZUZKSGhyNmNtMGZfTjRsOHFkLUxUTWMyUzRBbGx3RTRFZU5DQ1ZCODdZSXRTa0V6WmdyeUVqSHA4amw2NEtHNXNmVG1wdEFqOWRPSWlDei1Zcm10a1BvbzQwUi1kb3F6ZWdZeFNXbmV4RS1Gcm9YSkpmUmZBcUw4QnM?oc=5</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>7</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46054.54166666666</v>
+        <v>46055.44701388889</v>
       </c>
     </row>
     <row r="14">
@@ -866,24 +866,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Apollo appoints Valor as asset manager for logistics portfolio - Logistics Manager</t>
+          <t>Services - GIMA Day Conference 2026: the future of the supply chain for garden products - gardenforum.co.uk</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:21:00 GMT</t>
+          <t>Mon, 02 Feb 2026 12:04:40 GMT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOUUx3a255dUZramdIYndNZmxSMGkwVS1fSy12dW5FWUY5d1ltV0RGbF9jRjdBdldRVXA5RW1SVm9sWUF3emNaYW5QLU1hOWpfZlluX2dPZkxGQTZGdHMwVEJ1LW9WeWk1dHlZOHhsWkk3bTI1alhXRjkzUmlZdDJlaE56R1hrX2FHQ2VXTll2N3BzOElsSTk4alhrZng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPU3VFMUNRR1duajV0UmZPN3VTeklQYUF6VXlmbmc0RmdXOXpseW5Cd1FTdnBLNS1nQmoxbGNOQjEwWkp2RThUQUZLUlUyYVJwVnhKUFpzV1RPUkZwUDJHYTlpSnltdFNUaXlwT1cwMUpRVnFiVVhLcHFmczVMRUNmV19vbUZPWlg1SllsSTAzQm5HeG05X0NXWk1UVjlDQTd2NUlzaExVU2tLTlpYaHIzM2ZLLXpEQndfQmM4?oc=5</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>7</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46055.43125</v>
+        <v>46055.50324074074</v>
       </c>
     </row>
     <row r="15">
@@ -899,24 +899,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>China cuts tariffs on Scotch whisky - The Drinks Business</t>
+          <t>Price of consumer goods could surge as shipping costs soar, industry body says - The Guardian</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:56:37 GMT</t>
+          <t>Sun, 01 Feb 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPblMwMm5fMVJQejYzOWRYQ1BWWDhud0tfeTlIdnEzUEZYanRMbWdhQlhVNnprRGs0SVdjNjJtb2p4SUN1emU2ZnZBdl9HTVV6aFFvSUV4bWtsYTVnWjMyNzM3N0xQcVRWelpObUVQb0tUaE0tdkR5SGduMGhXWnpZWWF6SXU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNM2ZMdGRNWlRFaVVqVHg2Q0Q3X0c1Um5uRFEzRnJselR5czM5OXJZdHdCOVpnUGxtbXo3VUlTekowNkZMaEgyeEtBeDVDUEZfSXhyZG80NlQ4bFp1cnFwTVdCdURyRnk5Zzc0N2doM1BqSFBIY25Jb2dMdUhCclVTZV93XzNsQm9VN1R3VFY3ejB6eVQ4M1ZGRmI4SV9FdEhCcXI0VEdIQVAzVjV6bHBDdmNwZzlzd2c5OVpuNmVaa09vWmdFcjBKQkJn?oc=5</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>7</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46055.4559837963</v>
+        <v>46054.54166666666</v>
       </c>
     </row>
     <row r="16">
@@ -932,24 +932,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>NPA host Agricultural Supply Chain Adjudicator in Lincolnshire - National Pig Association</t>
+          <t>China cuts tariffs on Scotch whisky - The Drinks Business</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:49:27 GMT</t>
+          <t>Mon, 02 Feb 2026 10:56:37 GMT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOFBxVjc5ZFRKY2h4WHFMcmhnbWVBckZHNlpfVk9PVUhhREtMUldwMzd6c1hJUnZPZVRRRklRa1hHek14SHVvWGo0YmdVM1hxQ2g4cWFoNVo0Q2tRc0FUeUNsSnFFc3hXcnRqU2oxMTB4RmU4QkVWSFIxN2kyWjFhLVhPQk4xS3Q2Qk0wd1hXeVFxN1ZLVkxBbmhvVHZFTzJxV2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPblMwMm5fMVJQejYzOWRYQ1BWWDhud0tfeTlIdnEzUEZYanRMbWdhQlhVNnprRGs0SVdjNjJtb2p4SUN1emU2ZnZBdl9HTVV6aFFvSUV4bWtsYTVnWjMyNzM3N0xQcVRWelpObUVQb0tUaE0tdkR5SGduMGhXWnpZWWF6SXU?oc=5</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>7</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46055.45100694444</v>
+        <v>46055.4559837963</v>
       </c>
     </row>
     <row r="17">
@@ -965,24 +965,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Columbia Group appoints Prevention at Sea as compliance partner and rolls out MORSE platform across the fleet - shipmanagementinternational.com</t>
+          <t>NPA host Agricultural Supply Chain Adjudicator in Lincolnshire - National Pig Association</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
+          <t>Mon, 02 Feb 2026 10:49:27 GMT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxObWwwd0JPOVh6Rkp0cmFwckNxZ25TSThzZWtyS0N1dkRGOUV2ODBpUl82djNtZDROVVlmYUNibnpRUW5Cb2pvYnBWRGlLZk1xb2p6YVVqNXdsSWRRRTBFdDdPMWNpZ3JERDlvQzBkQy1qYU0tb2Q0MjQxcm9XZUlpdTc5aWR0OUxnbWV5QS13VDNxdkRMZ00wWm8wVlJENTBRdmZBR0k2dlVnSmNiRnVmZHFzRVktaTNXaU9FZWZ5YkthVHFkUndmWERXdFFYWjk3WU8zUXVFM2NPSlU2OWdDU2FLYXk3Y3NaekE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOFBxVjc5ZFRKY2h4WHFMcmhnbWVBckZHNlpfVk9PVUhhREtMUldwMzd6c1hJUnZPZVRRRklRa1hHek14SHVvWGo0YmdVM1hxQ2g4cWFoNVo0Q2tRc0FUeUNsSnFFc3hXcnRqU2oxMTB4RmU4QkVWSFIxN2kyWjFhLVhPQk4xS3Q2Qk0wd1hXeVFxN1ZLVkxBbmhvVHZFTzJxV2c?oc=5</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>7</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46055.44070601852</v>
+        <v>46055.45100694444</v>
       </c>
     </row>
     <row r="18">
@@ -998,24 +998,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mapletree on how European logistics is gaining momentum - Private Equity Real Estate | PERE</t>
+          <t>Columbia Group appoints Prevention at Sea as compliance partner and rolls out MORSE platform across the fleet - shipmanagementinternational.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 02:02:52 GMT</t>
+          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQbF9UQXJKSXljNU5GeW9JZmpVZ0ZobUNnTFF5bVFxanRIam4xX2lNMENFeTVJT1Z2WHF1bXI3WHphYXhfd0VQNWx1Z25UVy1WNkFKY0ZmY3hfYTAyYVhJanRnSW44M09CZ2lOcmRIc2czTnY2OVc3UlhFWjc5VGtSYng4QzNxbExj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxObWwwd0JPOVh6Rkp0cmFwckNxZ25TSThzZWtyS0N1dkRGOUV2ODBpUl82djNtZDROVVlmYUNibnpRUW5Cb2pvYnBWRGlLZk1xb2p6YVVqNXdsSWRRRTBFdDdPMWNpZ3JERDlvQzBkQy1qYU0tb2Q0MjQxcm9XZUlpdTc5aWR0OUxnbWV5QS13VDNxdkRMZ00wWm8wVlJENTBRdmZBR0k2dlVnSmNiRnVmZHFzRVktaTNXaU9FZWZ5YkthVHFkUndmWERXdFFYWjk3WU8zUXVFM2NPSlU2OWdDU2FLYXk3Y3NaekE?oc=5</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>7</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46055.08532407408</v>
+        <v>46055.44070601852</v>
       </c>
     </row>
     <row r="19">
@@ -1031,24 +1031,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Q&amp;A: Why 2026 is the Year the Supply Chain Takes Control - Supply Chain Digital Magazine</t>
+          <t>The North East’s Green Super Port: 18 months on, the opportunity remains vast - North East Bylines</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:46:41 GMT</t>
+          <t>Mon, 02 Feb 2026 08:12:00 GMT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQcm9wVVVGb0Mzc3M2WENybmx6VlVwQm9oY2RWMlZBRzZjaEF4UERWdkpmejZJWDJxaUZJXzAxb0hiVlpZQ29pVHh4SG9rcWhHa0RVdi1GMGZibTIxb1BkSVpLODNkbXZZcDlBM3puR0VjNUd6TzJ1UEhIN1hrX3NvVDRNOWs1TXZ2YjFnWC1xZDdZM0xyeVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOamgxNERESWJlUy11VUpyMHBVazQzM0tMUXpNRzY3UTk5bXBoV0x2bVZUMkxaUFl1YUFrS3NldGFfY2xuNy1jcjB0amc2UFR0cGlqWWlyQTFpVEVadkY4akJuU2FTeEF1M0FfMXgxejlrbVJvZDhpVFZEcVlVY1N4MFpBaGZnMm5ObmtxemxDWk41V0h4STExZ00wbEhuVWtJQkpha0pHLTI1VG9EdG5wXzBqbm5zY3E4dmpzbUlRekY?oc=5</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>7</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46055.36575231481</v>
+        <v>46055.34166666667</v>
       </c>
     </row>
     <row r="20">
@@ -1064,24 +1064,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The North East’s Green Super Port: 18 months on, the opportunity remains vast - North East Bylines</t>
+          <t>Mapletree on how European logistics is gaining momentum - Private Equity Real Estate | PERE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:12:00 GMT</t>
+          <t>Mon, 02 Feb 2026 02:02:52 GMT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOamgxNERESWJlUy11VUpyMHBVazQzM0tMUXpNRzY3UTk5bXBoV0x2bVZUMkxaUFl1YUFrS3NldGFfY2xuNy1jcjB0amc2UFR0cGlqWWlyQTFpVEVadkY4akJuU2FTeEF1M0FfMXgxejlrbVJvZDhpVFZEcVlVY1N4MFpBaGZnMm5ObmtxemxDWk41V0h4STExZ00wbEhuVWtJQkpha0pHLTI1VG9EdG5wXzBqbm5zY3E4dmpzbUlRekY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQbF9UQXJKSXljNU5GeW9JZmpVZ0ZobUNnTFF5bVFxanRIam4xX2lNMENFeTVJT1Z2WHF1bXI3WHphYXhfd0VQNWx1Z25UVy1WNkFKY0ZmY3hfYTAyYVhJanRnSW44M09CZ2lOcmRIc2czTnY2OVc3UlhFWjc5VGtSYng4QzNxbExj?oc=5</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>7</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46055.34166666667</v>
+        <v>46055.08532407408</v>
       </c>
     </row>
     <row r="21">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Clarion acquires Mountpark Chartres 2 - Logistics Manager</t>
+          <t>What are tariffs, how do they work and why is Trump using them? - BBC</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:31:48 GMT</t>
+          <t>Tue, 27 Jan 2026 10:32:09 GMT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9tY2V5UFFHU0pfb0hCa25JNHk5S0JWbXZadk5kU1ZKSWV3QzQtN05HRk5CeHBVeHpQYTdFSVR3UVVIcGVzczJxR2ZEa1dlWjlXcFNaT1E2enVuM0UyUldUai1iU25xSk1PT2NqLUFNWUpUTzI2a043ZHdSYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBweHdveUp5S2F0aGJwSEs2U2lOMkF6NzRNZTd3bEJUdTQwVjhRX0pjZmFzZ25hRzk4MHE0WW9KVkEtUjIxRUNWbXRzX3pmd1A5UWhyaE5Ja1ZWd9IBX0FVX3lxTE82Y0Q0dVVkNUhXb1o4Tkt6V1AycjA1dmkzbUs3d3JydDktMVNrSnNsNDI1Zk9BdmpMc1BQbGJneThSUDBmUkdUdFhDVTZaTTRGaGlwdDhnR3NPeXhDYW9F?oc=5</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>7</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46055.43875</v>
+        <v>46049.43899305556</v>
       </c>
     </row>
     <row r="23">
@@ -1163,24 +1163,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wallenius Wilhelmsen starts operating car terminal at Port of Gothenburg - Logistics Manager</t>
+          <t>Apollo appoints Valor as asset manager for logistics portfolio - Logistics Manager</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:24:18 GMT</t>
+          <t>Mon, 02 Feb 2026 10:21:00 GMT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOMzBjYXdWRGJ3QUN4QlgxWjJUeWUtVUxVSzhFbnRDOThwWFRySkJIZjNqUzNMRENVU0gxMzFlVUZqM1Y1dFFJQW9nbTlBQzdxVFdjazJ3XzdxWmgyZEVnblF5NnpscTZueVpuVnotU0Q0aUZTUW81aUM3dkFBSVNSMlMxQnduRUJZekxISnFmRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOUUx3a255dUZramdIYndNZmxSMGkwVS1fSy12dW5FWUY5d1ltV0RGbF9jRjdBdldRVXA5RW1SVm9sWUF3emNaYW5QLU1hOWpfZlluX2dPZkxGQTZGdHMwVEJ1LW9WeWk1dHlZOHhsWkk3bTI1alhXRjkzUmlZdDJlaE56R1hrX2FHQ2VXTll2N3BzOElsSTk4alhrZng?oc=5</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>7</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46055.391875</v>
+        <v>46055.43125</v>
       </c>
     </row>
     <row r="24">
@@ -1196,24 +1196,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>General Mills: Future-Proofing Sweet Corn Supply Chains - Supply Chain Digital Magazine</t>
+          <t>Clarion acquires Mountpark Chartres 2 - Logistics Manager</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:36:53 GMT</t>
+          <t>Mon, 02 Feb 2026 10:31:48 GMT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPSDNHaERCRzBmS2xTYWNEMUQ3UVdfejZycGRHcExYWHVOZm5LSllMVUE0ZElpcEhkd2czakpfbU5BbnowTFFKN1gyZzBZbkVxdWpVVVEzSFU3UFVfUUNnbERBTUF3VmM3Y2oxMG9KLUp5OUtHQU50alNTTmFCQ0ExVXBfcTNiSDR2eHM1X0JZbXFpQ3dN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9tY2V5UFFHU0pfb0hCa25JNHk5S0JWbXZadk5kU1ZKSWV3QzQtN05HRk5CeHBVeHpQYTdFSVR3UVVIcGVzczJxR2ZEa1dlWjlXcFNaT1E2enVuM0UyUldUai1iU25xSk1PT2NqLUFNWUpUTzI2a043ZHdSYw?oc=5</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>7</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46055.44228009259</v>
+        <v>46055.43875</v>
       </c>
     </row>
     <row r="25">
@@ -1229,24 +1229,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Why AI-native execution is the next step for supply chains - Logistics Manager</t>
+          <t>Wallenius Wilhelmsen starts operating car terminal at Port of Gothenburg - Logistics Manager</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:55 GMT</t>
+          <t>Mon, 02 Feb 2026 09:24:18 GMT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOSVEzSlZlTWE4QV9yZlM4QzVlN2pheHJsSjhVSlowVDJUUk9jaGRGT2psZ29OTUdpSENLNkE0VFQ4NjNvdFU4SjFlbXA2WU01M241WEhpMFBTSkxPSmJxTkxHU1pFN3A5SjJ2OEdvNHZRZV91RkZ3bjdDOUYyX2NyLUVaR3NDY3R0UjdtOWlPTDBROFZFZWVN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOMzBjYXdWRGJ3QUN4QlgxWjJUeWUtVUxVSzhFbnRDOThwWFRySkJIZjNqUzNMRENVU0gxMzFlVUZqM1Y1dFFJQW9nbTlBQzdxVFdjazJ3XzdxWmgyZEVnblF5NnpscTZueVpuVnotU0Q0aUZTUW81aUM3dkFBSVNSMlMxQnduRUJZekxISnFmRQ?oc=5</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>7</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46055.37563657408</v>
+        <v>46055.391875</v>
       </c>
     </row>
     <row r="26">
@@ -1262,24 +1262,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>China lifts sanctions on MPs and peers, as Starmer says he hopes Xi will visit UK - BBC</t>
+          <t>Why AI-native execution is the next step for supply chains - Logistics Manager</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 13:51:49 GMT</t>
+          <t>Mon, 02 Feb 2026 09:00:55 GMT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5lS2o5QUFSdzNFRFdORmdsd2hKMllEOUVhQ0MwUlp3eHEwSXR1UXlMXzlYZzRvOC1pcTJqSzV3amhQbFl1QU9ETzRWcGxIZy00SWRJVUxuMVRsUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOSVEzSlZlTWE4QV9yZlM4QzVlN2pheHJsSjhVSlowVDJUUk9jaGRGT2psZ29OTUdpSENLNkE0VFQ4NjNvdFU4SjFlbXA2WU01M241WEhpMFBTSkxPSmJxTkxHU1pFN3A5SjJ2OEdvNHZRZV91RkZ3bjdDOUYyX2NyLUVaR3NDY3R0UjdtOWlPTDBROFZFZWVN?oc=5</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>7</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46052.57765046296</v>
+        <v>46055.37563657408</v>
       </c>
     </row>
     <row r="27">
@@ -1295,24 +1295,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Net zero readiness in Hospitality, FMCG, Manufacturing, Logistics and Retail - theenergyst.com</t>
+          <t>General Mills: Future-Proofing Sweet Corn Supply Chains - Supply Chain Digital Magazine</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:46:56 GMT</t>
+          <t>Mon, 02 Feb 2026 10:36:53 GMT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPcENJelBLS2dmNFotWm5CLVpnY2h1dFhPbTlGYkJNZlRVSnVhNHJBZDFNU3lOMVNxWDRHc2NSYVpzZENlcEJaclRYNTB4TGhSNEM3b2RKMlA3TWxtN3NtMzFKaTNxWVNHUlowaVBGaTFHWnpQTlRSLS1SLW5tdTVJYjV5WjFtQnRodlg1R2V5dnNMWTJnNWlqT1o2al9pVUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPSDNHaERCRzBmS2xTYWNEMUQ3UVdfejZycGRHcExYWHVOZm5LSllMVUE0ZElpcEhkd2czakpfbU5BbnowTFFKN1gyZzBZbkVxdWpVVVEzSFU3UFVfUUNnbERBTUF3VmM3Y2oxMG9KLUp5OUtHQU50alNTTmFCQ0ExVXBfcTNiSDR2eHM1X0JZbXFpQ3dN?oc=5</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>7</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46055.44925925926</v>
+        <v>46055.44228009259</v>
       </c>
     </row>
     <row r="28">
@@ -1328,24 +1328,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The Compliance Inflection Point: Why Mid-Market US Insurers Are Feeling the Strain - Insurance Edge</t>
+          <t>Cargo outlook cools in 2026 as supply chain pressures persist - Air Cargo Week</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:02:57 GMT</t>
+          <t>Mon, 02 Feb 2026 11:42:00 GMT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOemlwSW5xR0c5TXk5ZXJtak96NktuWmpaUFRYcDZKWl9XMlg3dmJPLVZwOFVWQ0VuNFFUSWVSMEViZjhOZEpWbTZieXNVWjVwUW9QTGpucmVfQ2xDck55NEhsSzFhc2ItbjNmQkYzdkh4UE0xV05QLVFjM3hvc3BfTUZ3OGZsc1huVmFDVnhVWUVqVWFUc3NRUHN1VVZtRUZlcFZBcW9yTk9XU0l1aDBqX1JkNWRBYnJweW91MQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPdEo1Y2NzWUg1YW5pbXZqSUFfSC1WX3NCdTIwOS1HUnBCR01XNGIzVmJoZ1hMMWhydnhTeW1JRC01RFZEY2RoMGFHOGV0SmZDVF9IUW5kSGNYRXJsLUVGc05YSW1BYVY0bHktT0NTRGI4QWpxTFZNbXplaEtvT09veUFMT1phTDBXSmw1TExhMGo?oc=5</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>7</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46055.37704861111</v>
+        <v>46055.4875</v>
       </c>
     </row>
     <row r="29">
@@ -1361,24 +1361,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>How AMP8 digital compliance is shaping the water industry - Water Magazine</t>
+          <t>China lifts sanctions on MPs and peers, as Starmer says he hopes Xi will visit UK - BBC</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:05:04 GMT</t>
+          <t>Fri, 30 Jan 2026 13:51:49 GMT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNT2RfQVZPS1FHeHRURDhWalhPQU43d0RkOGFTTzRxd19BclVwRGtQMlJfUFB5TW5fY294SG13ajVWand6S2Z6a2FCaHFNcTFrQVNJQ0xIbWFOdkRhN2cxbGJ3aVRmVi1tNWt3WUxqUkxuUS1pYk8tWFh6N2ctbXlEYVRQUWd2SFhVNXZiMFVlclgzdkZUU2ZLSEpjdmpuVXpZV2dV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5lS2o5QUFSdzNFRFdORmdsd2hKMllEOUVhQ0MwUlp3eHEwSXR1UXlMXzlYZzRvOC1pcTJqSzV3amhQbFl1QU9ETzRWcGxIZy00SWRJVUxuMVRsUQ?oc=5</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>7</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46055.21185185185</v>
+        <v>46052.57765046296</v>
       </c>
     </row>
     <row r="30">
@@ -1394,24 +1394,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Skarv Shipping AS selects Oceanly Performance Plus to support automated data integration and digital fleet operations - shipmanagementinternational.com</t>
+          <t>How AMP8 digital compliance is shaping the water industry - Water Magazine</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
+          <t>Mon, 02 Feb 2026 05:05:04 GMT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQM2RvOWNMZ0JQblZOSjV3NHN3eldnckFLNldOaVc2cmU2YXRvakdmM2NhSlFXVmpmVnN3MFdrUjJqMGJxaWlXZFM4YVBPY2xBeXVETmVJYm9aMFNJdklfNmlkclNSbjc4X1BxcGluM1NVel9PN3R5VGNQVWJYVWw5T3ZfbjdhQ0UzdFI4QjFOOUs1M0JfNkY5cXVFN2hCNExaMTVBZG5XaW1rQ29MUG5waGdfQUs2OTV3TE9wVmdBeXN1VTUxSnd6NnNPOXBwYlNJS1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNT2RfQVZPS1FHeHRURDhWalhPQU43d0RkOGFTTzRxd19BclVwRGtQMlJfUFB5TW5fY294SG13ajVWand6S2Z6a2FCaHFNcTFrQVNJQ0xIbWFOdkRhN2cxbGJ3aVRmVi1tNWt3WUxqUkxuUS1pYk8tWFh6N2ctbXlEYVRQUWd2SFhVNXZiMFVlclgzdkZUU2ZLSEpjdmpuVXpZV2dV?oc=5</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>7</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46055.44070601852</v>
+        <v>46055.21185185185</v>
       </c>
     </row>
     <row r="31">
@@ -1427,24 +1427,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CEO of World’s Largest Container Shipping Company Says ‘No’ to Arctic Shipping - High North News</t>
+          <t>EU ready to impose sanctions on Kyrgyzstan — report - Eurasianet</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:50:10 GMT</t>
+          <t>Mon, 02 Feb 2026 09:56:19 GMT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQU1ZCNTRWdUhWN2VyUzZQbmlwSDFFNFlwckhWWVhMazdIR1lFQmhieUxBYjJzLWFUTmdsRkVXdFdndXlVWWtoSDNTUjFhUHBQMmQ0a2RVcVhwR0VmM0tpN1ZVTVlWNE5tV1RHVEZmdjNXa3JqQ3lRbmdOVnFGNndTM1FuX1lnU2p1alBuVTBxT1ppSmwtT2NUX1NETk1PVVN6M3dlSlFLNnMwdGVqWFU0elQxYWc4Z3lWVGVCQm9WQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTFBWb0tFRFFEc3BtZVhkUV94MWt2MUVzcGNMYmp3eGZHSmk4QmlyTC01U1VjU1JCQU9aM2dsVmMwYzMza1NfRmdHaEJKaGZiOXozMXM5bXVtRVJwb3JmbVhBaF9rRnQ3eTVLQ2lNUVgzcjB2NEI2U3dDX1VXazI?oc=5</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>7</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46055.45150462963</v>
+        <v>46055.4141087963</v>
       </c>
     </row>
     <row r="32">
@@ -1460,24 +1460,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Verdion plans €69m Greater Copenhagen urban logistics facility - Green Street News</t>
+          <t>Port of Tyne appoints new Direct of Innovation - porttechnology.org</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 07:45:57 GMT</t>
+          <t>Mon, 02 Feb 2026 11:45:34 GMT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOWU1GQkF6aWxiaWs2RjVoWTliVE9UcDRBOTE1aWJENE82amxXQXlmcTFpMERCUlUzckluZzA0N2paT09VeWhtVTU4YlpNZkticm8wWWs3UzZ1Q1BRcXA5bzVQd0tJRGJzVHUxdmdhMW4yOE5XNm1vclU3UUIydkkxdG11VDZmVnk3ak1ZZzNBdTNTeXBQTjhwcC1QMV9sMXJX?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNN05iX2doRUpwajRNSDFMVW1MUnU0d2VsOW1fbTdjR0V5Q1VkRzNHWlZwN1BkbV9SLXlYNF9ZNm1wb09YOUR0MU5jNXRTZHpnbWx0bkpsZWZfdTNiUDBOaW9CbWxxcWotZ3M4b2UtM0lseU1IdUpWaWpDaWpYTFRLeENqNjZhcEp4RzBj?oc=5</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>7</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46055.32357638889</v>
+        <v>46055.48997685185</v>
       </c>
     </row>
     <row r="33">
@@ -1493,24 +1493,24 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Panama voids Hong Kong-based firm's canal port contracts - BBC</t>
+          <t>Apollo Channels Billions Into AI Data Centers And Logistics Real Estate - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 13:16:05 GMT</t>
+          <t>Mon, 02 Feb 2026 11:05:44 GMT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFAyUDB1T0FCcGI3eV94eS1sRmdVbU1nMk5RdGtydFBzWDJlSWFTRGJQRTltbmd2UG9ZcjJLTnppZFF3b1ZjSTJQM0xfZkRKZ05iNmc2YmRDUVkyZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPLUozSE5oZTBTdVN1S1M5TW9SU3pIdUdKMHd1dy1rMi1CMEZsWW5xTXdid25DWEVMemx0UzFmUHZRcUpZOXQxeDFQY295NlVKQW96T2FBNkhCbjhSZTlyS05OQlhBbWIybG5qTk5BVklaS05xTFhZMWpuWVNtWV9vSFp5ekptV0dU?oc=5</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>7</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46052.55283564814</v>
+        <v>46055.46231481482</v>
       </c>
     </row>
     <row r="34">
@@ -1526,24 +1526,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>THIS WEEK: Russian sanctions, Ukrainian loan and US trade deal - EUobserver</t>
+          <t>Health and Safety at Scale - Logistics Business</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:00:55 GMT</t>
+          <t>Mon, 02 Feb 2026 11:15:24 GMT</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPZ0RuX1EzcDI4OVJDVTRMbmJMdTRuR3I0X3lDX1NYX3NBcUZDdEZIckxMMDhnYTNDMjhJM3A5UDE0UVpIUnV6clFYWkNOS1J5V3p2a1JkUGt6X19xWE5kZXcxeDB4QlZpNHBVRlJ2TTQ1Vmd2UF9qV1VybEhuME1HdnNMd0pNOVQ5cHlsV2hOUzVVVm9STGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQZVY5dHhMNlBKYnlkVmRxV1RlZ3hfdDV3T0FzQ1lTajZjaDAtSVV2RVlleUYxZWIxUDR2dXFhSEFtS1VGVy0yTnJQNVgtOERlNTJoWm5fVkFoaVJVajZiVXFhdS1WOFV2bFZKVl9IYjJkWURkWkxyWmxrM3BTQll2aHpn?oc=5</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>7</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46055.25063657408</v>
+        <v>46055.46902777778</v>
       </c>
     </row>
     <row r="35">
@@ -1559,24 +1559,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EU ready to impose sanctions on Kyrgyzstan — report - Eurasianet</t>
+          <t>THIS WEEK: Russian sanctions, Ukrainian loan and US trade deal - EUobserver</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:56:19 GMT</t>
+          <t>Mon, 02 Feb 2026 06:00:55 GMT</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTFBWb0tFRFFEc3BtZVhkUV94MWt2MUVzcGNMYmp3eGZHSmk4QmlyTC01U1VjU1JCQU9aM2dsVmMwYzMza1NfRmdHaEJKaGZiOXozMXM5bXVtRVJwb3JmbVhBaF9rRnQ3eTVLQ2lNUVgzcjB2NEI2U3dDX1VXazI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPZ0RuX1EzcDI4OVJDVTRMbmJMdTRuR3I0X3lDX1NYX3NBcUZDdEZIckxMMDhnYTNDMjhJM3A5UDE0UVpIUnV6clFYWkNOS1J5V3p2a1JkUGt6X19xWE5kZXcxeDB4QlZpNHBVRlJ2TTQ1Vmd2UF9qV1VybEhuME1HdnNMd0pNOVQ5cHlsV2hOUzVVVm9STGc?oc=5</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>7</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46055.4141087963</v>
+        <v>46055.25063657408</v>
       </c>
     </row>
     <row r="36">
@@ -1592,24 +1592,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Transfer deadline day: Follow text updates and watch Staffordshire &amp; Cheshire special - BBC</t>
+          <t>Net zero readiness in Hospitality, FMCG, Manufacturing, Logistics and Retail - theenergyst.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:43 GMT</t>
+          <t>Mon, 02 Feb 2026 10:46:56 GMT</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1NTld6YlRob0t1VEpvSzBLdEJ1UWJaS3J3RndGX2NRRUVjWWxway12aU5peHNXcHEyaXN4S3V5X3d5RXFOaWExdE43MXdJclI4X0l5cHFKOWNKZXY0QmZWeTRfQjg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPcENJelBLS2dmNFotWm5CLVpnY2h1dFhPbTlGYkJNZlRVSnVhNHJBZDFNU3lOMVNxWDRHc2NSYVpzZENlcEJaclRYNTB4TGhSNEM3b2RKMlA3TWxtN3NtMzFKaTNxWVNHUlowaVBGaTFHWnpQTlRSLS1SLW5tdTVJYjV5WjFtQnRodlg1R2V5dnNMWTJnNWlqT1o2al9pVUU?oc=5</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>7</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46055.37549768519</v>
+        <v>46055.44925925926</v>
       </c>
     </row>
     <row r="37">
@@ -1625,24 +1625,24 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Leyton Orient 0-1 Port Vale - BBC</t>
+          <t>Lamb welfare measures will be an “added cost” to supply chain, says NFU - Meat Management</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 17:03:00 GMT</t>
+          <t>Mon, 02 Feb 2026 11:56:09 GMT</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTFBFZ2R2eks5N1NhX0pmT1JnTEZJQjhSbmJJMUR5Zi1McWV4eVNMSmJWMk4ybDQwRmhJeVlWWml4dGVMOEdSS1pWWWM2MVBkWS1YRFdNVDhGbkltZGlqN09mRXJpc0g?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNYUVBWXIzNWlWWGRsbk1lVXE2RnVqMEtNbG9KR0YzbWlVTGJJNnpDaFN3YnRzMExRZlBESGxRem9mSXkxSEgySVpsSkxqM3pLSDFjNHdnckNmN2JtRGxFUWJYVTNYci00ZFdHbnE0bU5ZYUNVMmNGOEgxelc3cDJ4bXBVOGJGMlhOUlVhcGFWTkxLZjFUZU9wT2hOdk16Sl9XSmtpTkZYeXN6S0hDMVhSQzJrbW8?oc=5</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>7</v>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46053.71041666667</v>
+        <v>46055.49732638889</v>
       </c>
     </row>
     <row r="38">
@@ -1658,24 +1658,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>APMT open to temporary operation of Panama ports - porttechnology.org</t>
+          <t>The Compliance Inflection Point: Why Mid-Market US Insurers Are Feeling the Strain - Insurance Edge</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:55:34 GMT</t>
+          <t>Mon, 02 Feb 2026 09:02:57 GMT</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPYWNPVU9TXzUtb21BS2tJdEZPUkhfNFR5T29XRXBaX3llTkhwYVpQNFZPY0w3YUQ5NDktdVdPajNyc1F1Q1c2QTFOc1lqSlZpZWs2c1N2YmpDU1lTT3ZUeENDWnVrcmxnaDI4SzM4NGNEMGdVQ2paV21jLXg2NHIyMzlEZkdSVzZLTUdLZmFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOemlwSW5xR0c5TXk5ZXJtak96NktuWmpaUFRYcDZKWl9XMlg3dmJPLVZwOFVWQ0VuNFFUSWVSMEViZjhOZEpWbTZieXNVWjVwUW9QTGpucmVfQ2xDck55NEhsSzFhc2ItbjNmQkYzdkh4UE0xV05QLVFjM3hvc3BfTUZ3OGZsc1huVmFDVnhVWUVqVWFUc3NRUHN1VVZtRUZlcFZBcW9yTk9XU0l1aDBqX1JkNWRBYnJweW91MQ?oc=5</t>
         </is>
       </c>
       <c r="F38" t="n">
         <v>7</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46055.41358796296</v>
+        <v>46055.37704861111</v>
       </c>
     </row>
     <row r="39">
@@ -1691,24 +1691,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Transport NorthLink warns of seven days of disruption as freight sailings cancelled - Shetland News</t>
+          <t>Verdion plans €69m Greater Copenhagen urban logistics facility - Green Street News</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:31:32 GMT</t>
+          <t>Mon, 02 Feb 2026 07:45:57 GMT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNTUJsLUljdDNSNEx4SEFZWTc4TEFkaFFMZzg1ZUlJVEkyMGt0bXNIamlZcXlzSXk3YWVBMkZSZW1Na3hHaWxkVnRCNHVvVmlfV3RndkdxSGswaVcxVV9waWxCVlBTZmFQMlRrZ3R6UkphZHpycUdMQWpQYUpFaVZUU1pR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOWU1GQkF6aWxiaWs2RjVoWTliVE9UcDRBOTE1aWJENE82amxXQXlmcTFpMERCUlUzckluZzA0N2paT09VeWhtVTU4YlpNZkticm8wWWs3UzZ1Q1BRcXA5bzVQd0tJRGJzVHUxdmdhMW4yOE5XNm1vclU3UUIydkkxdG11VDZmVnk3ak1ZZzNBdTNTeXBQTjhwcC1QMV9sMXJX?oc=5</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>7</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46055.39689814814</v>
+        <v>46055.32357638889</v>
       </c>
     </row>
     <row r="40">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Norwegian court rules sanctions against Russian fishing firm Norebo are valid - SeafoodSource</t>
+          <t>Clarion Partners Europe acquires French logistics facility from Affinius - IPE Real Assets</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:51:44 GMT</t>
+          <t>Mon, 02 Feb 2026 11:33:47 GMT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQY3FfUTVqdHJrN0VGdXMtWjFmUE9UYWtLTzhabFlfLUw3OHRYMzlrZ1JOaWh6NC11LWxGSXk3QlZvb3lzVnBzNmlQVmdBNjZCeEsyeVV5VWNoUWR3dG5qNmNiNUFHeThrOEZkOUNtVGNEZjItTG1QT2xUN2VOYzJ0Vk1kQ2VpMGFqUF9DZTh6bUZhU1NzSVhTdkR4a3NNNFhEYkNEUnNPbW5nc3pvQ3FoRXRpd1lqQ3M1QXdIRUZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOS1g5VWhPM2VtR3lQSC1sVFRDNmhEVl9IdzYzWUw5QS1sVXgxZHhWc2o0bkR2WUtNTnlsUm45VnZiUV9ZVnlIeGdWbW1jbXhOYzViQlRxSEZtaHJoODQ1ZW96NHFHSWJtUGNqZC1xM1NVWnk4clcyT2VQSVhaRUtWRjdUQnlfWnZLOXM2dlFyaFNtWUQyYndCcDZTWHZXVnFLNWlRdV81NFdfWnUxcHVzMm1lb005R0FsM2g4aFJB?oc=5</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>7</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46055.45259259259</v>
+        <v>46055.48179398148</v>
       </c>
     </row>
     <row r="41">
@@ -1757,24 +1757,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Trump threatens tariffs on Canada planes and nations selling oil to Cuba - BBC</t>
+          <t>CEO of World’s Largest Container Shipping Company Says ‘No’ to Arctic Shipping - High North News</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 06:12:07 GMT</t>
+          <t>Mon, 02 Feb 2026 10:50:10 GMT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFB1WkVQc0puSWViS1UwYU43WVk1Wi1fcXZVa3hldVc5NE9kV1FZSjdjc0RfUUlieTZnVmJqWGxfcV8xR0pmWHU1dHR4UVRUV0hObkIxSkJQejIzUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQU1ZCNTRWdUhWN2VyUzZQbmlwSDFFNFlwckhWWVhMazdIR1lFQmhieUxBYjJzLWFUTmdsRkVXdFdndXlVWWtoSDNTUjFhUHBQMmQ0a2RVcVhwR0VmM0tpN1ZVTVlWNE5tV1RHVEZmdjNXa3JqQ3lRbmdOVnFGNndTM1FuX1lnU2p1alBuVTBxT1ppSmwtT2NUX1NETk1PVVN6M3dlSlFLNnMwdGVqWFU0elQxYWc4Z3lWVGVCQm9WQQ?oc=5</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>7</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46052.25841435185</v>
+        <v>46055.45150462963</v>
       </c>
     </row>
     <row r="42">
@@ -1790,24 +1790,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Trump tariffs live updates: EU, India seal trade deal in rebuff to Trump as he threatens S. Korea tariff boost - Yahoo Finance UK</t>
+          <t>Skarv Shipping AS selects Oceanly Performance Plus to support automated data integration and digital fleet operations - shipmanagementinternational.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Tue, 27 Jan 2026 16:42:00 GMT</t>
+          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPRzdWMzRXR1F4eUlpNzNLeGw0QzdFTkRhOFVqLTlubG03MEFqaEtqcHI5U2Nudm9OSm5vUmt3emVGVGVwX3NzZndFUExDY3B6OTBuVE1rUVFsakhxLVZwUW5Gal9pWUZUc19KMnNSSVpocmhHMGo4T1k5SGczanc2WkFteV9hVTRLdUhoVFNNSHZDVERpS1RHejZPTXRFNGlkTUlzS0JHWWdva3FQRnZFQkFLZUVodWZFbVlpRW9ILTliRUwxdHJIcGZ2aFhFbzBtOXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQM2RvOWNMZ0JQblZOSjV3NHN3eldnckFLNldOaVc2cmU2YXRvakdmM2NhSlFXVmpmVnN3MFdrUjJqMGJxaWlXZFM4YVBPY2xBeXVETmVJYm9aMFNJdklfNmlkclNSbjc4X1BxcGluM1NVel9PN3R5VGNQVWJYVWw5T3ZfbjdhQ0UzdFI4QjFOOUs1M0JfNkY5cXVFN2hCNExaMTVBZG5XaW1rQ29MUG5waGdfQUs2OTV3TE9wVmdBeXN1VTUxSnd6NnNPOXBwYlNJS1E?oc=5</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>7</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46049.69583333333</v>
+        <v>46055.44070601852</v>
       </c>
     </row>
     <row r="43">
@@ -1823,24 +1823,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>February strikes to hit Italian air, rail and port travel - VisaHQ</t>
+          <t>Panama voids Hong Kong-based firm's canal port contracts - BBC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 21:19:56 GMT</t>
+          <t>Fri, 30 Jan 2026 13:16:05 GMT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOMm0yN05jandUTjdrSVg5M2c3X0xTUGxPbTE5ZEJRSFlMZDRpLVJkandYUEJHSERIZmFQa1ZmaFFDc005ZDNYeU1kQ1VkNUI4QUZWWnZQY0xzazBxQU44UmlHcTg3NWFfdVd3MTV1MzZMMkdtWnVCZW1IdjQ3Ml8xSE9BVmYtbXFBVS1naVZWbktZa2dpbndXMHFWZFRuOWZJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFAyUDB1T0FCcGI3eV94eS1sRmdVbU1nMk5RdGtydFBzWDJlSWFTRGJQRTltbmd2UG9ZcjJLTnppZFF3b1ZjSTJQM0xfZkRKZ05iNmc2YmRDUVkyZw?oc=5</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>7</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46054.88884259259</v>
+        <v>46052.55283564814</v>
       </c>
     </row>
     <row r="44">
@@ -1856,24 +1856,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>What’s your duty of care? Moving the needle from compliance to strategy - Financial Reporter</t>
+          <t>Shipping investor J Lauritzen hires new head of research - Tradewinds News</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:00:24 GMT</t>
+          <t>Mon, 02 Feb 2026 11:03:44 GMT</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxOQWxzSlhrQUdiVFNXZUpEM0tHV1YtUUh5MjFYZHdGYTN6cFU5eFM0WGxxTlVDT3NMU01Wa1BGSGJPVFl1U2hhSUU4cFQzck9iOUVBeEpqV1JYaExWMFZROHRzUWhmc2p2dFlJeW9ZQU9aT1ZtdUZ6Um1VUjVKdmxFTF83NmZHRDNpSVA1YXRCVEJTTzJoaUhNaXFrM0NrVWg4X1U2dzVlTnFUbWhDa0RSRDREenoxOU0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNFZvNVlOdXhWeEVPakxtRTVVVkppb1ZmUjJmRW5mcGNsWkM3OWhpNW1IQldqVmx0VE9WSVlvc2N0TmloNDhHUUlQVlpPN1hzaGx0dkE2dmhqVURaNjU2U3ZyR1l5cnlfcHBCRVRzY0tiZEF1b2x1MjZQYXVDa25GdkVhZmhBOXEzUllVMHU5d0I5Ynl6WkJleWZQQ2ZjYUlhWk5qSHZTd2hRdWs?oc=5</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>7</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46055.41694444444</v>
+        <v>46055.46092592592</v>
       </c>
     </row>
     <row r="45">
@@ -1889,24 +1889,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Freightliner acquisition by CMA CGM completed - porttechnology.org</t>
+          <t>Abuja Pushes for a Modern Logistics Architecture - Air Cargo Week</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:45:34 GMT</t>
+          <t>Mon, 02 Feb 2026 12:13:26 GMT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxONmpqaUtvSnJHMGhhWUlBQ1hXdjJ4V25yTUZGMElZQ0NmNGdUODBFYmE0NThjUnl3UG1lbEZ2RVcxRDVlV0hvcmxPS3F1dDlFZExSY25lUkIyejBJTlRvSjFVZmU4R21zTHRaamRIY0c2ZHdMdzJfM3pqQWpkYTNHdEdUdmtBOXJ2ZXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1BZENaWFpKQldCdHo0UFpwTFZLdnBLYU5aZFc1TlhSaERkZGNrYVdXVk9KX0ppX0haX01lWUdRQjljV2pCVWFxamlnTmhpbWZTUGNyOGdRSUxWVTN4VlRUQXdYX3IxR2FIQkVrUHJoRzJQMXIxYTZNQTBwOV8wNGs?oc=5</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>7</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46055.44831018519</v>
+        <v>46055.5093287037</v>
       </c>
     </row>
     <row r="46">
@@ -1922,24 +1922,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Airbus Launchpad to boost UK space supply chain - Electronics Weekly</t>
+          <t>Leyton Orient 0-1 Port Vale - BBC</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:49:38 GMT</t>
+          <t>Sat, 31 Jan 2026 17:03:00 GMT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQOHVpMXdnT3FxOWVleG5CTnhsUTRMb0NuanFadkktRUJ3WXJWQ1lxcUdKYzRESVFNWFVNeXAwVDU1aEJ0STlQeHJpVUxBSXpDakRkME1PdXMwREJ5M2VJaV9uTXlDOGh5UnpRdlZVeGJscDlWNndjMVJBZ3d4RkV2TFVmelFXVU1IOFJHX05yeERtdmtaNUExY1YxUU5ZN1BDRFlTZVZrRFd0emktQi1GVmE3Szd2QTB4dEN5aVdtc3RvSktzSHlILVAyOHVjQlR2T3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTFBFZ2R2eks5N1NhX0pmT1JnTEZJQjhSbmJJMUR5Zi1McWV4eVNMSmJWMk4ybDQwRmhJeVlWWml4dGVMOEdSS1pWWWM2MVBkWS1YRFdNVDhGbkltZGlqN09mRXJpc0g?oc=5</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>7</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46055.2844675926</v>
+        <v>46053.71041666667</v>
       </c>
     </row>
     <row r="47">
@@ -1955,24 +1955,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Slough-based logistics firm DX Group boosts leadership team to support growth drive - Motor Transport</t>
+          <t>Trump threatens tariffs on Canada planes and nations selling oil to Cuba - BBC</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:57:19 GMT</t>
+          <t>Fri, 30 Jan 2026 06:12:07 GMT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOY1hqWUVQOU5fVG80QUNVMzFQRTNTUGZiclRDUUVPb0Y1OGpoSEttN21kaHVKM3cwcnNrNmxCNkNITnRUdDhIRVBla3pPbDU0WkE1bXdKRXNLWU5lTzhJdWZKMGdZVW1KOXlfUjRvUlNDTTUzNGxHUlpXN0dNVXJZdFJnUDZVWWtBd1diR3U0TC1LYl9OVmVwY3Y1T3Jqdl9VT0k3RWpiRENRbGhxQzNMWFhn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFB1WkVQc0puSWViS1UwYU43WVk1Wi1fcXZVa3hldVc5NE9kV1FZSjdjc0RfUUlieTZnVmJqWGxfcV8xR0pmWHU1dHR4UVRUV0hObkIxSkJQejIzUQ?oc=5</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>7</v>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46055.45646990741</v>
+        <v>46052.25841435185</v>
       </c>
     </row>
     <row r="48">
@@ -1988,24 +1988,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Building a logistics blueprint for precision therapies - Aviation Business News</t>
+          <t>Norwegian court rules sanctions against Russian fishing firm Norebo are valid - SeafoodSource</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:02:34 GMT</t>
+          <t>Mon, 02 Feb 2026 10:51:44 GMT</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxQSlI4Uk0zNDROcFZWanNtLXZkWWl5YmVIMUctd3VrQXRDVERJVUY5Tmx0OFkxUkJkQzBVLWg0d0VyRmdXbjJnSW5idGw0Wl93SnNnV1RqWDlqcmlCN0JkNGozcG9iWmp3bmRzVmhkSmQyVXBsaXRZWFVaQzNkQV9yVF9ERVpyZDJEN0JjSm5hdWtlZnp6RFBHNlRlVGZLRTdIZ3ppOHdnNjNWMGRhZFpZZnlUeG5CQmNjMnEwaHlhWGg3LTU0Y01jWmNzN1V6dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQY3FfUTVqdHJrN0VGdXMtWjFmUE9UYWtLTzhabFlfLUw3OHRYMzlrZ1JOaWh6NC11LWxGSXk3QlZvb3lzVnBzNmlQVmdBNjZCeEsyeVV5VWNoUWR3dG5qNmNiNUFHeThrOEZkOUNtVGNEZjItTG1QT2xUN2VOYzJ0Vk1kQ2VpMGFqUF9DZTh6bUZhU1NzSVhTdkR4a3NNNFhEYkNEUnNPbW5nc3pvQ3FoRXRpd1lqQ3M1QXdIRUZR?oc=5</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>7</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46055.25178240741</v>
+        <v>46055.45259259259</v>
       </c>
     </row>
     <row r="49">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Port Houston marks record year for container volumes - porttechnology.org</t>
+          <t>APMT open to temporary operation of Panama ports - porttechnology.org</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQTndhNFdMREF2R3NaN0VidFZKWFNGZmNVWWd2bHMwaEE1NjB2R3Rsc3hZR2lFYy1EUThMSzJ0SWZPNk5hSkNMTmlZUTlUelpKX3JScXNDUG5yeHZtWGFyYkR1dFY4VGtSWDBodmpDMTR3Ym1rUlAyYUdwYkRvZnM3djNETVZoSllLeDJfaHdVUzFSRzQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPYWNPVU9TXzUtb21BS2tJdEZPUkhfNFR5T29XRXBaX3llTkhwYVpQNFZPY0w3YUQ5NDktdVdPajNyc1F1Q1c2QTFOc1lqSlZpZWs2c1N2YmpDU1lTT3ZUeENDWnVrcmxnaDI4SzM4NGNEMGdVQ2paV21jLXg2NHIyMzlEZkdSVzZLTUdLZmFR?oc=5</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -2054,24 +2054,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Morocco’s fresh produce, fast and reliable across the sea - Fruitnet</t>
+          <t>Trump tariffs live updates: EU, India seal trade deal in rebuff to Trump as he threatens S. Korea tariff boost - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:27:17 GMT</t>
+          <t>Tue, 27 Jan 2026 16:42:00 GMT</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPTWdXNzNubDc4TERZRmo1WHJfNEhKS3B4UFNUc2h0cUJSZU5jSEo5NE1Zdy1IUEgydnJaQVRYZkEwajNhcnBZcmZzVXFyaFJlUFl3SVlZMGFJdWM1bWtYWU5rdXY2QzJJR3BrbFhtcy1uY2FXT2lDbUVrZHZvY3hXekFiQm1kdUdSdXJIR3Bzc2ZTNTZtVVVEMFJXZDFVUzBPS1lvQ21CUHg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPRzdWMzRXR1F4eUlpNzNLeGw0QzdFTkRhOFVqLTlubG03MEFqaEtqcHI5U2Nudm9OSm5vUmt3emVGVGVwX3NzZndFUExDY3B6OTBuVE1rUVFsakhxLVZwUW5Gal9pWUZUc19KMnNSSVpocmhHMGo4T1k5SGczanc2WkFteV9hVTRLdUhoVFNNSHZDVERpS1RHejZPTXRFNGlkTUlzS0JHWWdva3FQRnZFQkFLZUVodWZFbVlpRW9ILTliRUwxdHJIcGZ2aFhFbzBtOXc?oc=5</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>7</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46055.35228009259</v>
+        <v>46049.69583333333</v>
       </c>
     </row>
     <row r="51">
@@ -2087,24 +2087,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Acwa signs deal to ship green ammonia from giant 4GW Saudi project to German port - Hydrogen Insight</t>
+          <t>Transport NorthLink warns of seven days of disruption as freight sailings cancelled - Shetland News</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:57:19 GMT</t>
+          <t>Mon, 02 Feb 2026 09:31:32 GMT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNaUVnQmE1cEVxck1WZWF0dlA5bkFKOEpsc21XWHc3U1hIakI5X1VsLWtEMjNSRFlJZ0VNbHo4SkZsRGRwdWUxOXhsMnVNVDB2RFBOZmQwLWotWC1kTlR6R0RnRzhaVUx6Nmg2M0dBUmVoSFdUSklJZ0ZSTldmb3JPU05rWS1SZ1lkbHRUZTZka09raXJRNnlXbjg1b181bjEtTkZCX29ZMHpMWUhHeHRKWG1TYUdMcF9obnFud0JIcXE0dm40YTN3TUlGZDd2cm5Yenc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNTUJsLUljdDNSNEx4SEFZWTc4TEFkaFFMZzg1ZUlJVEkyMGt0bXNIamlZcXlzSXk3YWVBMkZSZW1Na3hHaWxkVnRCNHVvVmlfV3RndkdxSGswaVcxVV9waWxCVlBTZmFQMlRrZ3R6UkphZHpycUdMQWpQYUpFaVZUU1pR?oc=5</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>7</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46055.41480324074</v>
+        <v>46055.39689814814</v>
       </c>
     </row>
     <row r="52">
@@ -2120,90 +2120,90 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Exclusive | Maritime Regulator’s New Head Targets Global Risks to Shipping - The Wall Street Journal</t>
+          <t>Crystal International unveils advanced logistics hub in China - Just Style</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:30:00 GMT</t>
+          <t>Mon, 02 Feb 2026 10:57:30 GMT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgNBVV95cUxQS2c1ZUlCRlpZSFhIcjRha0h4cVhUOHRYaUtCa3RRaUVDT2ZGU0lVQjFVdTBGbThCR0pGZzdiRkhTd0ZsWUpyNTBKY19QekMwdWJ5bDNMM2lJQWtYTm5TNmJoUndYMVIwZUdUS05ZQ3c0YktfN2Fnb1Y5OWpyRVRfelgtVzc5ZDRrQ1BxekJ5RFFzY1B3dGh2b001UVRxenJJcEd6bmVxMWJuZUdUUFZ5ZldzZlNxS2c2Y1d3UDZyVWxpUDZpUS02aWdFQWlGWndRSFFsQU1UcjN4OUlXbnlCdTF0SnBPaU5xNlRwZmhZajhmZFFrcHhveVJ2akJXOThwVHRkY3p5NnhDTG9QZEtHbVlsb3lvcDUwOElMNUtuVlUxVm5ST2U1Vk1jbi1FNTRlUUZmMWxndTdPRnA3VThsUTBHcmNOb1RpZGR5WjlpY3JzWnZsXzJSd2lQNFRWRnR4bE5zUEJwRFlRMUg4aXJyTmN0MmsyM1hCcHVSQUhXVGRTSmlXNE5LbFBWWndlb0ZRYi1ySTFubGFvWTRBbkhkbDlSQldodw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBTLVJYX3pEcmhvNzAwR2tNVUZjQmJGbk54SVpwLVhxOGVrQ1A3NmtfY2NlTFY1Z0Jwdzd6QzhQN19QTnI5Y1h6N3RHUWZNczFDNlVCZXdaQVlSRXhsaTN5N0VSMjY3QUxtWWh3cDA1djRROVd2ME5nQWZjb2dUUVU?oc=5</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>7</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46055.4375</v>
+        <v>46055.45659722222</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Protest</t>
+          <t>Supply_Chain</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Metropolitan Police strikes called off as workers accept new pay offer - Unite the Union</t>
+          <t>Freightliner acquisition by CMA CGM completed - porttechnology.org</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Thu, 29 Jan 2026 09:40:32 GMT</t>
+          <t>Mon, 02 Feb 2026 10:45:34 GMT</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPZGZLQ1JjVFFWRWJFa01lWUhfRkhfOGd5M3Z6SGRuQUxPcmkwR1N1M3ZYSmxUdjMwRnByb3ViOG1fdGJuS2Uycm1DUDJsNmpFVjJNZEMyU2pyZ1NnREI3dUxVaEIwMk1pSTM4ak5ULXpYZnRtVzFqNEVnSHpPbWpWeFNrOGxfVlAydE9wLWxBTmU0WkY5WEdDeUJ2LUF0MjVnRTc0VWpGZi1SOTVQZ0o0bzRWVW5Ua1FZbjhIM29Sa3p5Q1ZIRE5oOFJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxONmpqaUtvSnJHMGhhWUlBQ1hXdjJ4V25yTUZGMElZQ0NmNGdUODBFYmE0NThjUnl3UG1lbEZ2RVcxRDVlV0hvcmxPS3F1dDlFZExSY25lUkIyejBJTlRvSjFVZmU4R21zTHRaamRIY0c2ZHdMdzJfM3pqQWpkYTNHdEdUdmtBOXJ2ZXc?oc=5</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>7</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46051.40314814815</v>
+        <v>46055.44831018519</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Protest</t>
+          <t>Supply_Chain</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
+          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Italian government to meet after clashes in Turin injure over 100 officers - Anadolu Ajansı</t>
+          <t>Pakistan head to T20 World Cup amid sanctions threat after India match boycott call - The Independent</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 16:17:04 GMT</t>
+          <t>Mon, 02 Feb 2026 11:51:00 GMT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxORXF6SmMtNXN1WVVNNW56U09wbC1IY2tteWN0SkVGUU1vZmlYSjhZek1VUWRxVEJQcDg0S09lTmtpVm4zMFdUSWtDMUYteFBDc1BxUUx1azJkNzhMc3dOZW0zOEdpSVV1NWRMdXdqb3BTTWFWVC1ORk5JcEN1MFd3VGZ6WWd5NjBUeGlyQjQxNkdBNDFkdjU1UjRVTzFVSF9lSE5McUJKVzVvdXdZRjRiN2ZxT08?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPRHM4VWxaMFVOLVg1VjRNWGI3ME1HV283eFA0Ri1SZkJud19vdVRTMzZhZWM1eGljWjNPQkZuUHRsOWRkVi1QdXU5Y0V3eHZsdXdsYnJ4bHRwY0M2XzIycTZDVlVnYXUyWUlKRlBjVURtNDdncnlHOVpoVklxRlFiUkxZOFFUNU8wcklGb3IxX095eXUzd3dsQ0FR?oc=5</t>
         </is>
       </c>
       <c r="F54" t="n">
         <v>7</v>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46054.67851851852</v>
+        <v>46055.49375</v>
       </c>
     </row>
     <row r="55">
@@ -2219,24 +2219,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Children and police officers among at least 30 killed in Israeli strikes on Gaza - The Guardian</t>
+          <t>Metropolitan Police strikes called off as workers accept new pay offer - Unite the Union</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 07:33:00 GMT</t>
+          <t>Thu, 29 Jan 2026 09:40:32 GMT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPYzV0Y0xxR2lTSU85dzc3TW1wYkVJSzhzQzY3bGRLQ1hsVXpZR0tOeHR5Y2cwRzhZZ3lRT1U1OHZIX3ZyUklUQjE5bllRSF9BWENDMVJ4WDhudTJBTXZYeTlqUmtjbDhkT2N3Y0RvZ19WSkxRckdTWXFQSGw4NE1LNm1UNUVNai1jS3FsRERaeEh5NURYN1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPZGZLQ1JjVFFWRWJFa01lWUhfRkhfOGd5M3Z6SGRuQUxPcmkwR1N1M3ZYSmxUdjMwRnByb3ViOG1fdGJuS2Uycm1DUDJsNmpFVjJNZEMyU2pyZ1NnREI3dUxVaEIwMk1pSTM4ak5ULXpYZnRtVzFqNEVnSHpPbWpWeFNrOGxfVlAydE9wLWxBTmU0WkY5WEdDeUJ2LUF0MjVnRTc0VWpGZi1SOTVQZ0o0bzRWVW5Ua1FZbjhIM29Sa3p5Q1ZIRE5oOFJ3?oc=5</t>
         </is>
       </c>
       <c r="F55" t="n">
         <v>7</v>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46053.31458333333</v>
+        <v>46051.40314814815</v>
       </c>
     </row>
     <row r="56">
@@ -2252,24 +2252,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sussex Police panel says it has "lost confidence" in PCC - BBC</t>
+          <t>Update after police called to convenience store - Cambs Times</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 17:19:01 GMT</t>
+          <t>Mon, 02 Feb 2026 11:04:00 GMT</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5pSmI0TlhZN3pPMGxjaUIybEp3VUJQU1lWQ014Ykg1TEVCa1d5aGFLSDhlTHZzYXY1SHJLLWcxMGI2eEFlWlhwZnpGVnZYSFpfWFA3THYyWFJjZG5N?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxORnRnWW9xTkxDMVVISlZvNjZVS0RfZGhhLUU4RFBNZVNsbmExOEJZZHVBZ1IzelZXVl9nOGZFZGQwcTFfaE1YZjlUODVJWExsXzNiVm5DMnpQNGM4RHplZXZRZG5HMHNjaE1VY0VjOGdpd194cU1rUmMzQ3NXV0QyWXBoQkYzMEVVM1A2eFU3VlpkYTA?oc=5</t>
         </is>
       </c>
       <c r="F56" t="n">
         <v>7</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46052.72153935185</v>
+        <v>46055.46111111111</v>
       </c>
     </row>
     <row r="57">
@@ -2285,24 +2285,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Police probe launched after jewellery thieves strike at vulnerable Smethwick woman's home - Express &amp; Star</t>
+          <t>Iranian police detain four unspecified foreigners over unrest - Reuters</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:11:04 GMT</t>
+          <t>Mon, 02 Feb 2026 11:29:03 GMT</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNSGdYOGR4YWRSQ0pFc0VxSUdoc3RNUkZ3bXRvdDBuVDBBWWhYLS0td1lPVmtDUWYwZGpqbVZ5RkxrMWQ4SkRqWHhBSkFjWll4QU11cnZKMEtRWTRmNi1xOWRsWTlnSmtkSXN6MVZRT2hCZHBnR2dlbmV1NzZBcWJ5SnJZcDJWNWtENVFkdVNKa2wyRTFkLVJRWDJTSHg2MlZUUDNWY0xOcFBuTkpWUUdRZG0xZzkyeGstTkdVMHF0UGo0UVlzYmNfdGQzMFVKNUtvMHF3UlpRSmJhR211YWFJQTdZVFFXSDJRU1lWNXQwQmxFQjNFMHk0VnFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbEFYWUliVTVUN0ZCdEdQYVNQQWl2VUJqakF3S19nbG1BMjE2M2xDa1NLRXI3U1pjVFRsWGZhRUFfMnQ5cjdPTmF3VFlpcENfenhkOTFWOXhMckdETkVINWNaY3RCMWxwTElDVzg0U2xLamVuSXlVQXJ0RmpNb25taUp1aEFJc19IRXdhZk9DZHE5OVQzSnR5LVM5QmdhZFNHT2dPY2ZvNDVPSlhTdVRLdjJZMldiZkZaTzFsSA?oc=5</t>
         </is>
       </c>
       <c r="F57" t="n">
         <v>7</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46055.34101851852</v>
+        <v>46055.47850694445</v>
       </c>
     </row>
     <row r="58">
@@ -2318,24 +2318,24 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Police and crime commissioner storms out of hearing after being censured for joining anti-migrant protests in Crowborough - GB News</t>
+          <t>Another e-scooter taken into police possession - Fenland Citizen</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 15:14:07 GMT</t>
+          <t>Mon, 02 Feb 2026 11:33:00 GMT</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPNzRfSWt4cFdoY3NpZmJoN3JicjVvcThEaHRCWTdtZW9CUWxNOEVNMURnV05DQ2hGUmJlbUwzbTg1OVZBTkJJaHBZc3dRMUNqTm5rQXBQeDQyMWFIQnh5bHJNWURBeTBJd1Q3OWJzMmNNeVZtbFg4NnZlX0QzQVRNZTdxUThmcjZONG4yaUU0SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQY0xxNnhKTTZwdUtJdVZNZXBSQ0lwUlpxMDhCUWxhUFBFLXpUaDJMNmF2OW1YY2hWSTJ5Zm1Vbk9mcDl5UjZpWm1Jd1FPYW1mVk5sZV9xc3dlYktqRWlOQTFaUDBBU0JGMVhQZnRkSkMwYV9QWnpsY0RQU1VtRlhWWnJDb0o5WkIyWlZNcTVoTHZvM25keS1BRg?oc=5</t>
         </is>
       </c>
       <c r="F58" t="n">
         <v>7</v>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46054.63480324074</v>
+        <v>46055.48125</v>
       </c>
     </row>
     <row r="59">
@@ -2351,24 +2351,24 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Iran prosecutor says police contained unrest without weapons - ایران اینترنشنال</t>
+          <t>Children and police officers among at least 30 killed in Israeli strikes on Gaza - The Guardian</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 11:48:43 GMT</t>
+          <t>Sat, 31 Jan 2026 07:33:00 GMT</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTFBiSERLckdhME9CS3BkUHRiZ2YtUERZOXl1ZE8yX0RCSTlDT2R1TjlsdktQem8tNENHZkRMNkxISmJSTmRYMzUyT0VCbDhkRlVuaWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPYzV0Y0xxR2lTSU85dzc3TW1wYkVJSzhzQzY3bGRLQ1hsVXpZR0tOeHR5Y2cwRzhZZ3lRT1U1OHZIX3ZyUklUQjE5bllRSF9BWENDMVJ4WDhudTJBTXZYeTlqUmtjbDhkT2N3Y0RvZ19WSkxRckdTWXFQSGw4NE1LNm1UNUVNai1jS3FsRERaeEh5NURYN1E?oc=5</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>7</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46054.49216435185</v>
+        <v>46053.31458333333</v>
       </c>
     </row>
     <row r="60">
@@ -2384,24 +2384,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Police brace as pro-Palestine and Ukip rallies descend on capital - London Evening Standard</t>
+          <t>Italian government to meet after clashes in Turin injure over 100 officers - Anadolu Ajansı</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 16:01:16 GMT</t>
+          <t>Sun, 01 Feb 2026 16:17:04 GMT</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNTmtKeW9taDV6aVJQZkp6ZG45aTNoaE9QMWxDM2o0bmdXTWZYakoySThLamgzMDA1bG84TnhjS2pZdFhncDV4N1Y2MVhnWUMtNV9TN1lPMExhMzFqNXVPeFpCMk1kRHNZTjJETmF4OEFnZ25ETi1XZVhuNWNTUGY4eTFVS2VKQlpCOFY4WkVJb2FoT2JJWkVjVGphT29idF93Zlpnd2ZfQ3FmYU12c18tbXR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxORXF6SmMtNXN1WVVNNW56U09wbC1IY2tteWN0SkVGUU1vZmlYSjhZek1VUWRxVEJQcDg0S09lTmtpVm4zMFdUSWtDMUYteFBDc1BxUUx1azJkNzhMc3dOZW0zOEdpSVV1NWRMdXdqb3BTTWFWVC1ORk5JcEN1MFd3VGZ6WWd5NjBUeGlyQjQxNkdBNDFkdjU1UjRVTzFVSF9lSE5McUJKVzVvdXdZRjRiN2ZxT08?oc=5</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>7</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46053.6675462963</v>
+        <v>46054.67851851852</v>
       </c>
     </row>
     <row r="61">
@@ -2417,24 +2417,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Herts police appeal for information after burglars strike in Bishop’s Stortford - Bishop's Stortford Independent</t>
+          <t>Sussex Police panel says it has "lost confidence" in PCC - BBC</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 14:59:00 GMT</t>
+          <t>Fri, 30 Jan 2026 17:19:01 GMT</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNclZROGF1SmltZGNncGt2VUhoa0E5YURxSngtZ0NwVGZuWk9jajBUSkRyS1NXUGhIYzJvem1nMzNjeHIyTlJzTjRRUWhGT2QwV3dpNEJkN2tZdml3dmc4dnFYWWFSbGx0TWhWa0cxRk1raEV3ekdneTJVTklwa1lKZFRvSDNUdERuaGRZaEhmVmI5X1lQUEF0aXZRLWFvdHliNmVlNTJTYUJHNGo0M2xJcklzaVp0b19IMXlUbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5pSmI0TlhZN3pPMGxjaUIybEp3VUJQU1lWQ014Ykg1TEVCa1d5aGFLSDhlTHZzYXY1SHJLLWcxMGI2eEFlWlhwZnpGVnZYSFpfWFA3THYyWFJjZG5N?oc=5</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>7</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46052.62430555555</v>
+        <v>46052.72153935185</v>
       </c>
     </row>
     <row r="62">
@@ -2450,24 +2450,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Thousands turn out for national rallies in support of French police force - RFI</t>
+          <t>Police probe launched after jewellery thieves strike at vulnerable Smethwick woman's home - Express &amp; Star</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 15:32:04 GMT</t>
+          <t>Mon, 02 Feb 2026 08:11:04 GMT</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOeVFhWDVkaDhlV3hzZUF1SGh5VzdFMWJCNW9MbGJMLVZ1M25vS2FfX0x6NHV6ZXBJd2ZoSnhpX0dVQkJfNFp0b2drZ3ZzMXlXaXVVbWQxc2Z3R1VwUWIxNVotaWtfaDdrcUR4M0VpcUxrc281cmdSdjhWbjE4ZU1XTl9xUGI5UEVwR0lROXcwZkRwTUtkdEd2Ti1kRGx4WHNwZHBHa3JRZ2NOYUVLQ2pLdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNSGdYOGR4YWRSQ0pFc0VxSUdoc3RNUkZ3bXRvdDBuVDBBWWhYLS0td1lPVmtDUWYwZGpqbVZ5RkxrMWQ4SkRqWHhBSkFjWll4QU11cnZKMEtRWTRmNi1xOWRsWTlnSmtkSXN6MVZRT2hCZHBnR2dlbmV1NzZBcWJ5SnJZcDJWNWtENVFkdVNKa2wyRTFkLVJRWDJTSHg2MlZUUDNWY0xOcFBuTkpWUUdRZG0xZzkyeGstTkdVMHF0UGo0UVlzYmNfdGQzMFVKNUtvMHF3UlpRSmJhR211YWFJQTdZVFFXSDJRU1lWNXQwQmxFQjNFMHk0VnFB?oc=5</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>7</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46053.64726851852</v>
+        <v>46055.34101851852</v>
       </c>
     </row>
     <row r="63">
@@ -2483,24 +2483,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Clime Capital Announces March Quarter Dividend Guidance Of 1.35 AU Cents Per Share - TradingView</t>
+          <t>Police and crime commissioner storms out of hearing after being censured for joining anti-migrant protests in Crowborough - GB News</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 01:59:00 GMT</t>
+          <t>Sun, 01 Feb 2026 15:14:07 GMT</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPaERFNTN6UzRGZkxwdHJpTzVWdm0yOEgzM083aFUwVnZXbEpYbFg2cTFndjF5a2xSX1lFdzBkb3h1TGhIODRfcWh6dUIxdnJJbTFURTQ5dnJxVjFOVHhoZk41dHlrd1VDMi00VWpuSURqaWVQYVBZTHhrV1BFMVBnMkM4NEJVNExLenEycGUwYVBMU0ZldGE3Z2x3SGd2UUtOLXJDX01VYmpJYmNDMTJBcmNuWk9GUnphbHRranNOWWVfbGd1VlZBb1U4cWFmRXJVQWpWdDBEQXd2RVFrN2pTbTNhU2NXXzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPNzRfSWt4cFdoY3NpZmJoN3JicjVvcThEaHRCWTdtZW9CUWxNOEVNMURnV05DQ2hGUmJlbUwzbTg1OVZBTkJJaHBZc3dRMUNqTm5rQXBQeDQyMWFIQnh5bHJNWURBeTBJd1Q3OWJzMmNNeVZtbFg4NnZlX0QzQVRNZTdxUThmcjZONG4yaUU0SQ?oc=5</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>7</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46055.08263888889</v>
+        <v>46054.63480324074</v>
       </c>
     </row>
     <row r="64">
@@ -2516,24 +2516,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PPB Monitors Protest Activity, No Arrests Made - City of Portland, Oregon (.gov)</t>
+          <t>Police brace as pro-Palestine and Ukip rallies descend on capital - London Evening Standard</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 08:17:17 GMT</t>
+          <t>Sat, 31 Jan 2026 16:01:16 GMT</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNZEFueFNUZzJZLVlBWWtONDlJdzJuZTNFcUMta2M2SXA4bC12MHpJX1NhRFdVLXMyRWJCNUE3OU5NOUgtejVNRTk0V21ueW1fYUV3WGJIT1J4c0gwV2Q5TUdjY0h4dTJ5V2VNYzdGVXVxZlJKdFNNZEMzbXlNYUgyQXZEa3Mxc0xFbUNxcy1CUVhOejBXYkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNTmtKeW9taDV6aVJQZkp6ZG45aTNoaE9QMWxDM2o0bmdXTWZYakoySThLamgzMDA1bG84TnhjS2pZdFhncDV4N1Y2MVhnWUMtNV9TN1lPMExhMzFqNXVPeFpCMk1kRHNZTjJETmF4OEFnZ25ETi1XZVhuNWNTUGY4eTFVS2VKQlpCOFY4WkVJb2FoT2JJWkVjVGphT29idF93Zlpnd2ZfQ3FmYU12c18tbXR3?oc=5</t>
         </is>
       </c>
       <c r="F64" t="n">
         <v>7</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46054.34533564815</v>
+        <v>46053.6675462963</v>
       </c>
     </row>
     <row r="65">
@@ -2549,24 +2549,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Palestinians inspect the site of an Israeli strike on a Hamas police station in Gaza City - Reuters Connect</t>
+          <t>Herts police appeal for information after burglars strike in Bishop’s Stortford - Bishop's Stortford Independent</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 11:05:00 GMT</t>
+          <t>Fri, 30 Jan 2026 14:59:00 GMT</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxOR3JoaXRwOWp3MTJYUFMxWl9GUm83WWdEaTE1cTdQWFJKdkxOamhURFUybVdUTVZvaW5UcHdtcC11VXZkNnU3a29QUDVLdFZwWElTZW53dUVwazJlMVVaaVhoeEJMb0xuY25KUkVham5Db2EtRm1nRGdNb0Q1WXR4aFV0Q1dnOVdSRFFxSHFOQmQ1bUxtQ0J5TS0wMExNa3JJZFY1RXVvSm5KNjdqWkNXT1hyLVNfTWQySzY5c2cyVWpNc0pVWVB6bE9tNjdCUnZld1UzeE1iczgyZlczbGlqYkdDNm5kMU52bE8tdE5WMlZYOFJDX1pkY0otUmtuNm01YWFTRWJjTTNaMHJ2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNclZROGF1SmltZGNncGt2VUhoa0E5YURxSngtZ0NwVGZuWk9jajBUSkRyS1NXUGhIYzJvem1nMzNjeHIyTlJzTjRRUWhGT2QwV3dpNEJkN2tZdml3dmc4dnFYWWFSbGx0TWhWa0cxRk1raEV3ekdneTJVTklwa1lKZFRvSDNUdERuaGRZaEhmVmI5X1lQUEF0aXZRLWFvdHliNmVlNTJTYUJHNGo0M2xJcklzaVp0b19IMXlUbg?oc=5</t>
         </is>
       </c>
       <c r="F65" t="n">
         <v>7</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46053.46180555555</v>
+        <v>46052.62430555555</v>
       </c>
     </row>
     <row r="66">
@@ -2582,24 +2582,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Man sought by police after thief strikes at North Yorkshire shop - The York Press</t>
+          <t>Thousands turn out for national rallies in support of French police force - RFI</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 15:15:55 GMT</t>
+          <t>Sat, 31 Jan 2026 15:32:04 GMT</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPTndPZmlBeWVlWkk5VEdjb3FfeV9jSGRQQUotV2dZdlJVOURaNlo2a2tSRkFSYTdlUGZOUWZnRnc3dl9hN09WUVU1ZE40RzZiNnhNeEswaTk2a1g5TVMxRjFmUl9UdndTLTh6ci1kXzhPQnhpV2cxQUVaV0xjWU8xazlmTG42Q2R3LU5NNk1mSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOeVFhWDVkaDhlV3hzZUF1SGh5VzdFMWJCNW9MbGJMLVZ1M25vS2FfX0x6NHV6ZXBJd2ZoSnhpX0dVQkJfNFp0b2drZ3ZzMXlXaXVVbWQxc2Z3R1VwUWIxNVotaWtfaDdrcUR4M0VpcUxrc281cmdSdjhWbjE4ZU1XTl9xUGI5UEVwR0lROXcwZkRwTUtkdEd2Ti1kRGx4WHNwZHBHa3JRZ2NOYUVLQ2pLdA?oc=5</t>
         </is>
       </c>
       <c r="F66" t="n">
         <v>7</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46053.63605324074</v>
+        <v>46053.64726851852</v>
       </c>
     </row>
     <row r="67">
@@ -2615,24 +2615,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Exclusive: Police Agency Weighs Non-Face-to-Face Protest Reporting After Rulings - 조선일보</t>
+          <t>Eight Arrests made at Demonstration, including Three for Assaulting Police, Queen Street West and Bay Street area (Mahnoor Mohyuddin, Jennifer Vong, Kyle Stephens, Woodrow Fraser-Boychuk, Abe Berglas, Darcy Belanger, Bryn Williams &amp; Charles Kaake - Reddit</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 22:50:33 GMT</t>
+          <t>Mon, 02 Feb 2026 12:33:10 GMT</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOUzZGcXNNdUJLYVFaV3VNYWR2ZmRwcDV1eEhUMXktUDdvMFhLYXRVU1VpVWM5Q2Q1WVN5UHY5aVI3cGtadkotRmpsS3hOdWFxNlpGWjJiZFdxRWtiVVhQSDRicGxyZGx1SnZXNXNmR3VDNXRicEJVaG55LXk4cjlON29hTGMyWFho?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYlA1UmFxRnlZNXpJODk5X0hOWldUOElDdG1mVXhndl93LUhackpTa1FYZDBjRWR1dmFhc2xrYXMzMFo4WV94OEtZb0ZpYTljNlJYb0RVd1llS0RuWmRHRlA4QUFJaG5QTzBzaDRKUFBBUWNDR1pDdklZUXBvdnVqMmJiMVZydUp1Q0hVV2IydDZQY0F6eGtYdXB1M0w5QU8weWVEag?oc=5</t>
         </is>
       </c>
       <c r="F67" t="n">
         <v>7</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46054.95177083334</v>
+        <v>46055.52303240741</v>
       </c>
     </row>
     <row r="68">
@@ -2648,24 +2648,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Haredi soldier caught in anti-draft protest saved by police - The Jerusalem Post</t>
+          <t>Clime Capital Announces March Quarter Dividend Guidance Of 1.35 AU Cents Per Share - TradingView</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 01:58:48 GMT</t>
+          <t>Mon, 02 Feb 2026 01:59:00 GMT</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5xTDZ2R0tKT2N0WmtaUlluNHI5UXpTMjVQeDZodHR1RFNfdERpbjB0eVNiby0tYVJQTDZvbGtpTlRBWWRhQ0dzc2llSERUaEc4VUE4V2pZYmNpa2FpN3B4YjZoZ2ZZbjZOSmF3bzJkVTVWZGJWOXlqYmJvYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPaERFNTN6UzRGZkxwdHJpTzVWdm0yOEgzM083aFUwVnZXbEpYbFg2cTFndjF5a2xSX1lFdzBkb3h1TGhIODRfcWh6dUIxdnJJbTFURTQ5dnJxVjFOVHhoZk41dHlrd1VDMi00VWpuSURqaWVQYVBZTHhrV1BFMVBnMkM4NEJVNExLenEycGUwYVBMU0ZldGE3Z2x3SGd2UUtOLXJDX01VYmpJYmNDMTJBcmNuWk9GUnphbHRranNOWWVfbGd1VlZBb1U4cWFmRXJVQWpWdDBEQXd2RVFrN2pTbTNhU2NXXzA?oc=5</t>
         </is>
       </c>
       <c r="F68" t="n">
         <v>7</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46054.0825</v>
+        <v>46055.08263888889</v>
       </c>
     </row>
     <row r="69">
@@ -2681,123 +2681,123 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Mayor of Portland, Oregon, demands ICE leave the city after federal agents gas protesters - Politico</t>
+          <t>Man sought by police after thief strikes at North Yorkshire shop - gazetteherald.co.uk</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 22:29:52 GMT</t>
+          <t>Sat, 31 Jan 2026 15:15:55 GMT</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOaU1ISXJEUElQZXpNOWxJVTBSOFpiaVREZl9WajBTUXFGbzZtbjV4UnBjM01mc1pqdnJzRU9ZZEtEVS15N0dfTkRnUjRZRk9KMENsRlVUanY4aGw5WnRFb09MNDBCZmNXbDAwNzF0MXowU0tFS0dXQ28tdzV6ZkljRHI3cjNteWZ6aTU3YXZyTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNbm9JWXBPWWJPeG5FaWFVUnk5V1A4U1R6V182OFd2QWZtNzlaZWljd213Z1ZxTm1iR25hRmpvd2hpX1BhNFZpcUpxeGZObGNPb0h4S1lfeExRQnBjTnhITEh3N2pmenZKUWtaNWtmQmJPNXIwaDFZdi1VSXpWZnNSNnU4cFItZjhYVmVVRTNqVWh2TDky?oc=5</t>
         </is>
       </c>
       <c r="F69" t="n">
         <v>7</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46054.93740740741</v>
+        <v>46053.63605324074</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Technology and human rights - Amnesty International UK</t>
+          <t>PPB Monitors Protest Activity, No Arrests Made - City of Portland, Oregon (.gov)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:19:47 GMT</t>
+          <t>Sun, 01 Feb 2026 08:17:17 GMT</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPNHlIOVVoNVd4VmE2V3B1b0JLemxfMTcyYXQxakg2Q0dLekxWLW1nS3Myb3BnNk1TUm9Va1BzR3dSdE93SlRmV2gxN1ZoNmFKSm1YSGF3NUVQOG5qMi1mdnp4WHVBeXJ1MTlrWE42ZkhCaHp1cmhXQlMwMkd4czhaczJXWmxMT0Raa1JKbjhSZy1uUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNZEFueFNUZzJZLVlBWWtONDlJdzJuZTNFcUMta2M2SXA4bC12MHpJX1NhRFdVLXMyRWJCNUE3OU5NOUgtejVNRTk0V21ueW1fYUV3WGJIT1J4c0gwV2Q5TUdjY0h4dTJ5V2VNYzdGVXVxZlJKdFNNZEMzbXlNYUgyQXZEa3Mxc0xFbUNxcy1CUVhOejBXYkE?oc=5</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>7</v>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46055.43040509259</v>
+        <v>46054.34533564815</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NHS trials AI and robotics to speed up lung cancer diagnosis - UKAuthority</t>
+          <t>Haredi soldier caught in anti-draft protest saved by police - The Jerusalem Post</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:01:03 GMT</t>
+          <t>Sun, 01 Feb 2026 01:58:48 GMT</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNVW9sb25UeG1CVzdNOGVXWFRsT1ZBYWhwYkVTYkRZT0E3SURaNHdxeko1ejh5S2xnQThQaWp3TjRrOHM1TE1GcmxXcWFvMWZleFpRZVRNeWpQZW9fZXdBOVZjZTVJTjlUb01YTkRsZWZEQmdheTJ5d2ItdUt4b0JPX3RvZGZWc2JWZU5NRjVSbzNzQlF1Q0JabXRtemtYQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5xTDZ2R0tKT2N0WmtaUlluNHI5UXpTMjVQeDZodHR1RFNfdERpbjB0eVNiby0tYVJQTDZvbGtpTlRBWWRhQ0dzc2llSERUaEc4VUE4V2pZYmNpa2FpN3B4YjZoZ2ZZbjZOSmF3bzJkVTVWZGJWOXlqYmJvYw?oc=5</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>7</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46055.3340625</v>
+        <v>46054.0825</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Why banks shouldn’t wait for AI to fix the Gen problem - Retail Banker International</t>
+          <t>Planned NLC protest: FCT Police urge rescheduling in public interest - Vanguard News</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:28:04 GMT</t>
+          <t>Mon, 02 Feb 2026 11:26:31 GMT</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPNkJaSEM4djg2STlSalNWM0c3MmhmS1ZNS1c5MG14VUREZzNha25fVXp3VXF0YUczMkRlMEwtVldORHU4TFA1dEtLY3dfeXpmcW5UbHJLR09mX3FYZlFwbmtCbU1GZ3lsMFBUZmhpU2ZHMzlVZUxkSG0wNkRCeFcwQkk1OW5ZUlVaNXFPVktQb1g0djI5ZkQzU0ZKTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPNko1V2d1Szh2NWV0NDFpVDBjVE1XQlRPbjFvWnU4ekhma1dJUWp5TUdXRVdSM1BxUlNBZmY3MUNZakpFbkRFTFI0Mk5jVGVnc1Z0eWpPV2lFZXZycFNQUG1teW5TNktZdXVncVIxRVdSTHJOeGhnT2RGY1BEQlkyZXlkYVFjVEdKcjhmSHMwUzVCU2ZER2VIT3ZWc1k4c3BBUEFNSmRuQdIBrAFBVV95cUxPakFWT2JzSEE0djhXNUJXZDBaeTNTamk0RDM0a0R1WGVlcVQ0dnBodDhlOWI4RllNNlRISVZISWR2aGd0OXo0RE9xVzFZSElHaFluRTRYcVJ2em9BVlFyZFRxMG9jYWRYQktSQU5iaXBQWUItaFBlbFVyWGRxdGJqNVlua1VqQ3RzMTZqbGQzZS1XWURLcGVWbjhIQlhSZ3NUOGRGaEthSl90RXl3?oc=5</t>
         </is>
       </c>
       <c r="F72" t="n">
         <v>7</v>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46055.39449074074</v>
+        <v>46055.47674768518</v>
       </c>
     </row>
     <row r="73">
@@ -2813,24 +2813,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>AI and tech adoption in treasury - Private Funds CFO</t>
+          <t>Dow to replace 4,500 jobs with automation and AI as shares decline - Packaging Europe</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 02:00:49 GMT</t>
+          <t>Mon, 02 Feb 2026 11:08:32 GMT</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE9HX2wxTWg4OXVDNHpST0Z0MGZsRVJZVkVRSHJyWVJKMmk2QVN1Rk9LQmdfSjF1a0h1Vy1tSEpyREJpajlEcWRjZFdYRlZiT1ltYk0wb3hHUm1GejByQ183dTJWMlFXQmVOdDdyVGpjU2lVOFU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPUG85LWpVTTB1ajhzU3dMMEtCa3NkMDRxbmpjZTV4RmlvZ1dpSlh2VmZZSW40VEV2QzcwTDVaQVltdnpKT0gya19GT3I1VnJFUGNjRkNGNUtobGFCS0RjV2x1NmV5YTQ3bzlYUWxHRl81dnpLVk1vVHlEemtUU0JDeDk0SVhDYXBsSG9pMXBJdnJfOWpPQ3U4NjNVWm1IeEhCT1l6aWUxQ09EaGg0czl5MXh3?oc=5</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>7</v>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46055.08390046296</v>
+        <v>46055.46425925926</v>
       </c>
     </row>
     <row r="74">
@@ -2846,24 +2846,24 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>IFR position paper on AI in robotics released - International Federation of Robotics</t>
+          <t>Technology and human rights - Amnesty International UK</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:50:47 GMT</t>
+          <t>Mon, 02 Feb 2026 10:19:47 GMT</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1uM2Vnek8zdm5IV1hWem9CYWl1S0czMEJLd3lhNHNlLURxajlQZy1ISzdSd28yblRfeUpKV3ZsYWlPYlJsNGdDalFWMUQyOTVqSmQxMzNqV1Y2SE9UbzRxcjc3RzVRcTc0NG9tYV9JbU5fWVAzemRVMTVhV1o?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPNHlIOVVoNVd4VmE2V3B1b0JLemxfMTcyYXQxakg2Q0dLekxWLW1nS3Myb3BnNk1TUm9Va1BzR3dSdE93SlRmV2gxN1ZoNmFKSm1YSGF3NUVQOG5qMi1mdnp4WHVBeXJ1MTlrWE42ZkhCaHp1cmhXQlMwMkd4czhaczJXWmxMT0Raa1JKbjhSZy1uUQ?oc=5</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>7</v>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46055.4102662037</v>
+        <v>46055.43040509259</v>
       </c>
     </row>
     <row r="75">
@@ -2879,24 +2879,24 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Abusers using AI and digital tech to attack and control women, charity warns | Violence against women and girls - The Guardian</t>
+          <t>The Telecoms.com Podcast: Ericsson, AI and Nokia - Telecoms</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 19:12:00 GMT</t>
+          <t>Mon, 02 Feb 2026 12:28:13 GMT</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNalRlb3UyM2w2eHBJQjRDYjNIMmN5Yl9sSDlRRmVDOUdpS0N5b3BHR0RXanJwM1FNd3pGWGw5T1RRYWZJQU9pOGluSUM2V2QxaDVyU3lJTVl1WS1OdzZlbGFQZG9YYzhENldpSy1lM2RrMFB4V01NVlRvUS1aLVpSY2QxTjk0YlN0M1ZuRGFwOURVQWoyQWo2MWdsRTVsY2xmZ0gtVUc4UzJTSXc2V3ZpV1o2YUVRUHc5Y1hSYkd3LWo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPTHhsYVpnTHdHNkNEQXR5YTVXeEdDSFh2dE9YLTJsdVdFbDV6MkxuQzJ5Q0xTdEZFb2VaMjlESi1JZDU1QWJpekR4ZExxY196ekhkZ2lJUDZzMnp5MjFrS250eDh5OGRSckRLczFKdjJKYVcyQlhmdEtSWTA2R0VLTTZUa1dhV2dlYXc?oc=5</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>7</v>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46052.8</v>
+        <v>46055.5195949074</v>
       </c>
     </row>
     <row r="76">
@@ -2912,24 +2912,24 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>How sustainable funds are navigating AI, defence and financials - Trustnet</t>
+          <t>NHS trials AI and robotics to speed up lung cancer diagnosis - UKAuthority</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:01:33 GMT</t>
+          <t>Mon, 02 Feb 2026 08:01:03 GMT</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRktGQTJJdXpHeldsX3E3NEl3ckx2QjkxU2tIb3lPUF84dEI0a2ZfQjVjbTNMeHpZUFZjdkR2bldWTnpMRmNjMnBkNFZ5Rk05dW5xeEpsTWo1YkRXUjhpYkdEYS1od0dPSmhScjZPRjZsYVBxTzlUbXh1QlVrbVhwaFRyNTB4aEk4V2I3b1dhV1J4VC1vRUdsMmdTUEFFeElqbE1J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNVW9sb25UeG1CVzdNOGVXWFRsT1ZBYWhwYkVTYkRZT0E3SURaNHdxeko1ejh5S2xnQThQaWp3TjRrOHM1TE1GcmxXcWFvMWZleFpRZVRNeWpQZW9fZXdBOVZjZTVJTjlUb01YTkRsZWZEQmdheTJ5d2ItdUt4b0JPX3RvZGZWc2JWZU5NRjVSbzNzQlF1Q0JabXRtemtYQQ?oc=5</t>
         </is>
       </c>
       <c r="F76" t="n">
         <v>7</v>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46055.45940972222</v>
+        <v>46055.3340625</v>
       </c>
     </row>
     <row r="77">
@@ -2945,24 +2945,24 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Vera van der Burg puts AI and ceramics into "reflective" feedback loop - Dezeen</t>
+          <t>Why banks shouldn’t wait for AI to fix the Gen problem - Retail Banker International</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 09:28:04 GMT</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTE5RNF82VUc5cDNNTzhsdHpwbXB6TDBhNW80M2k2Y0NRbFlRYzdoV21GTDNEcko5UDdjbmxIVkgyeHhNWkRCLVJ0SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPNkJaSEM4djg2STlSalNWM0c3MmhmS1ZNS1c5MG14VUREZzNha25fVXp3VXF0YUczMkRlMEwtVldORHU4TFA1dEtLY3dfeXpmcW5UbHJLR09mX3FYZlFwbmtCbU1GZ3lsMFBUZmhpU2ZHMzlVZUxkSG0wNkRCeFcwQkk1OW5ZUlVaNXFPVktQb1g0djI5ZkQzU0ZKTQ?oc=5</t>
         </is>
       </c>
       <c r="F77" t="n">
         <v>7</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46055.375</v>
+        <v>46055.39449074074</v>
       </c>
     </row>
     <row r="78">
@@ -2978,24 +2978,24 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AI 'slop' is transforming social media - and there's a backlash - BBC</t>
+          <t>AI and tech adoption in treasury - Private Funds CFO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:54:06 GMT</t>
+          <t>Mon, 02 Feb 2026 02:00:49 GMT</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9wNDA2bFFUbmx5aDlVcjdxaWE1c1JHZDZTcmxnampFRW5PN19EejRhQklPMkJmeDNYZnlMczE3MWl0M0h2UkhpZUN5b0hoX0RRZzExcTBZUmV3d9IBX0FVX3lxTE9LZjR2U0dKMjJ1WktUTy1JaWFWUkluMWYtSmJBQ0J4QmVuTVhhTUZTUGN5eUZ5UDdGMFZLeHN2TWNPaHZPSGk4LUtlYkpuYVA1Vk9Gd0p3RThuWTNrYXM4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE9HX2wxTWg4OXVDNHpST0Z0MGZsRVJZVkVRSHJyWVJKMmk2QVN1Rk9LQmdfSjF1a0h1Vy1tSEpyREJpajlEcWRjZFdYRlZiT1ltYk0wb3hHUm1GejByQ183dTJWMlFXQmVOdDdyVGpjU2lVOFU?oc=5</t>
         </is>
       </c>
       <c r="F78" t="n">
         <v>7</v>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46055.28756944444</v>
+        <v>46055.08390046296</v>
       </c>
     </row>
     <row r="79">
@@ -3011,24 +3011,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>“A cloud-enabled, digitally resilient Europe transforms the protection of its citizens, infrastructure and strategic interests” - Thales Group</t>
+          <t>IFR position paper on AI in robotics released - International Federation of Robotics</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:08:42 GMT</t>
+          <t>Mon, 02 Feb 2026 09:50:47 GMT</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQc3lvdXNHRWx4aTVFNFlPbGUyTjB5UlVaN3dhSUhvbXQ5dmF1Tk91REd1QTU4R2VPbGc0b0VEbTZrRlE0cHJWaXVFYmlXaDFDMDhqM3BUOWtNZzJLb0FBSEh3T2pwLWEyTE5ycEpEX19mSmJ4TG40UTIzRVdZTk1IdEpFaWpfVmtoZFRTaXRBREk1YzdNdk1NOVJFRHpzdTJPemlFYmZiWGtuWEJJWVgyaVlDSDBsRjFoaVVUU2tjLU9ZUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1uM2Vnek8zdm5IV1hWem9CYWl1S0czMEJLd3lhNHNlLURxajlQZy1ISzdSd28yblRfeUpKV3ZsYWlPYlJsNGdDalFWMUQyOTVqSmQxMzNqV1Y2SE9UbzRxcjc3RzVRcTc0NG9tYV9JbU5fWVAzemRVMTVhV1o?oc=5</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>7</v>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46055.38104166667</v>
+        <v>46055.4102662037</v>
       </c>
     </row>
     <row r="80">
@@ -3044,24 +3044,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>EU Selects SUPREME Consortium to Develop The Union’s Superconducting Technology - The Quantum Insider</t>
+          <t>How sustainable funds are navigating AI, defence and financials - Trustnet</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:24:45 GMT</t>
+          <t>Mon, 02 Feb 2026 11:01:33 GMT</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNaUNORlkxWXBCMW5YVjZIdHFFck9Yc2VhbGxWMElvaTI2RW01azg1cDBJTWlaclpXZENadEVsNXZiRnNpdUt3QjE5UkVkclByTTNEVXowa1VlTGZ0RlVIaWVIVkwzcjB6b1RVeTlkcjlWMXJrU2psMnNCbm1Fdkg0cW9faGpkVjFZNk1UVE1WejhXTjRfaHdaSUstY0k0UWZjeXNLYWJkbF9SUFRTWm9ZZTNXQ2VaQThROXlFXw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRktGQTJJdXpHeldsX3E3NEl3ckx2QjkxU2tIb3lPUF84dEI0a2ZfQjVjbTNMeHpZUFZjdkR2bldWTnpMRmNjMnBkNFZ5Rk05dW5xeEpsTWo1YkRXUjhpYkdEYS1od0dPSmhScjZPRjZsYVBxTzlUbXh1QlVrbVhwaFRyNTB4aEk4V2I3b1dhV1J4VC1vRUdsMmdTUEFFeElqbE1J?oc=5</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>7</v>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46055.3921875</v>
+        <v>46055.45940972222</v>
       </c>
     </row>
     <row r="81">
@@ -3077,24 +3077,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>UPS Resets Network To Favour Automation And Higher Margin Deliveries - Yahoo Finance UK</t>
+          <t>Abusers using AI and digital tech to attack and control women, charity warns | Violence against women and girls - The Guardian</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 01:06:00 GMT</t>
+          <t>Fri, 30 Jan 2026 19:12:00 GMT</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNaVo5eHdfOGZhUjJoM0RQeTBpbWNDb0NkdnZKclhQcWtCc2NJUGFmTVBZQmNwcFdibW9QY2JfVjVMTDRiMjNWRkxaU1VPd2hYOWlZSS1GUlJjWFlGMjBfVWZETUVBaUNsUENXVkJ4eDVBNVN6Y2dkNFRVSzBPQXc4dkFqZXNPR2d3QVV4SWRB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNalRlb3UyM2w2eHBJQjRDYjNIMmN5Yl9sSDlRRmVDOUdpS0N5b3BHR0RXanJwM1FNd3pGWGw5T1RRYWZJQU9pOGluSUM2V2QxaDVyU3lJTVl1WS1OdzZlbGFQZG9YYzhENldpSy1lM2RrMFB4V01NVlRvUS1aLVpSY2QxTjk0YlN0M1ZuRGFwOURVQWoyQWo2MWdsRTVsY2xmZ0gtVUc4UzJTSXc2V3ZpV1o2YUVRUHc5Y1hSYkd3LWo?oc=5</t>
         </is>
       </c>
       <c r="F81" t="n">
         <v>7</v>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46055.04583333333</v>
+        <v>46052.8</v>
       </c>
     </row>
     <row r="82">
@@ -3110,24 +3110,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Betting blind on AI and the scientific mind - The Transmitter</t>
+          <t>AI 'slop' is transforming social media - and there's a backlash - BBC</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:00:58 GMT</t>
+          <t>Mon, 02 Feb 2026 06:54:06 GMT</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNdWJUT1lZS2tZZEVHXzlBbUJOaVl3Y2VLa3dXblRNcmxsci16YnBrWENIanhRRHFoY1k5VmkyenF6VzdXaGEtRW9WVFlwSXhtTFVHLTdLb1RGVTY0Y2dhZ3dWOHdPZDB1SWFNZnZoR0UyN05TNzQxYmx6eG9QRHROZERYX24tRVg0d0NKTm1OT1RRNU1WUTE0b21zT09UTW04?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9wNDA2bFFUbmx5aDlVcjdxaWE1c1JHZDZTcmxnampFRW5PN19EejRhQklPMkJmeDNYZnlMczE3MWl0M0h2UkhpZUN5b0hoX0RRZzExcTBZUmV3d9IBX0FVX3lxTE9LZjR2U0dKMjJ1WktUTy1JaWFWUkluMWYtSmJBQ0J4QmVuTVhhTUZTUGN5eUZ5UDdGMFZLeHN2TWNPaHZPSGk4LUtlYkpuYVA1Vk9Gd0p3RThuWTNrYXM4?oc=5</t>
         </is>
       </c>
       <c r="F82" t="n">
         <v>7</v>
       </c>
       <c r="G82" s="1" t="n">
-        <v>46055.20900462963</v>
+        <v>46055.28756944444</v>
       </c>
     </row>
     <row r="83">
@@ -3143,24 +3143,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Maxio Report suggests B2B SaaS and AI growth remains strong but has become more selective - Enterprise Times</t>
+          <t>Vera van der Burg puts AI and ceramics into "reflective" feedback loop - Dezeen</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 07:14:23 GMT</t>
+          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxQS1Y4c09NU1JsSUlBMjFudjlEUGlkX19mdWR6Wm5pZ3VpV0NMd0JFTjY4YmtPd1VqWjRzb2E3aGNyMjlxSlBUVm5aMnl5Z1RabC1rNEZpcW1mSURYaUZVVko5dUNkQ2kzekltTDR4dHpTQS1uZFFHN2hWYS0zYnl1NEp5UERRczJwU2pKUnkzakN3c3RZaXM2R3EwX0tXZWgxcUlVRmRwOTc4OGxacmRWbjM3WXNQaUNYcnhwOXptTXpHU2RpRWpNaVEwUEU1UzZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTE5RNF82VUc5cDNNTzhsdHpwbXB6TDBhNW80M2k2Y0NRbFlRYzdoV21GTDNEcko5UDdjbmxIVkgyeHhNWkRCLVJ0SQ?oc=5</t>
         </is>
       </c>
       <c r="F83" t="n">
         <v>7</v>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46055.30165509259</v>
+        <v>46055.375</v>
       </c>
     </row>
     <row r="84">
@@ -3176,24 +3176,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Microsoft Q2 2026 Earnings: Can AI and Cloud Keep CX Ahead of the Curve? - CX Today</t>
+          <t>“A cloud-enabled, digitally resilient Europe transforms the protection of its citizens, infrastructure and strategic interests” - Thales Group</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:46:47 GMT</t>
+          <t>Mon, 02 Feb 2026 09:08:42 GMT</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNUC1EZDJEcjROV0lVNzhneHVKWXk5NEcxZHk3OVZ5ellocGZJUnpTbHI2ZmNBbDVYY19SbS1XWGotdC1ISzE1S3RiT3dqWEFBY0JpUzlndDRCRlJ5SmdfZ2JhSlZQMUJsLUQ5UHA4NGZ3dlVKYmlRbnN6akZKSWZMbWxPWGtOOEVfZ24tMHBNMmZCam5ZeFhlRkkxd001SS1qanpXanNWM2xQQjNVaTRaV2Rvb0hLQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQc3lvdXNHRWx4aTVFNFlPbGUyTjB5UlVaN3dhSUhvbXQ5dmF1Tk91REd1QTU4R2VPbGc0b0VEbTZrRlE0cHJWaXVFYmlXaDFDMDhqM3BUOWtNZzJLb0FBSEh3T2pwLWEyTE5ycEpEX19mSmJ4TG40UTIzRVdZTk1IdEpFaWpfVmtoZFRTaXRBREk1YzdNdk1NOVJFRHpzdTJPemlFYmZiWGtuWEJJWVgyaVlDSDBsRjFoaVVUU2tjLU9ZUQ?oc=5</t>
         </is>
       </c>
       <c r="F84" t="n">
         <v>7</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46055.4491550926</v>
+        <v>46055.38104166667</v>
       </c>
     </row>
     <row r="85">
@@ -3209,24 +3209,24 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Grok, AI and “free speech” – Starmer vs Musk - palatinate.org.uk</t>
+          <t>AI deepfakes are reshaping cyber risk – and insurance must keep pace - Insurance Business</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 20:30:01 GMT</t>
+          <t>Mon, 02 Feb 2026 11:25:07 GMT</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE9Qa2J6bG5BUjIzZ2k0Zkl6Ynk4a0x3dl9Hbm1yenJMNE1iUFM1cVY4d0hUcmdwYk5XRTB5a3ZjN0h6eldTVU41TkdWV185ZzFLQ0VCZkdkVU9keFZubF9kV0ZsQUdteE5jdDlKdHRpdUdjNXRacVpwMDR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNd0JwN0R2S2lhZk02UGFIVWlwODVoZ0NQZTMxZzFURWZURExNbmpXRFlfemNZTWpwNXFidktkSDlSek1EYzlmZzlRSGxoN1dxeG9vcmZYbS1PNU5qTld2RVNQZUNwMXlKcnROQUFXYmtmQUdoVUxxNmV2VlVDRnBSMEZtam1MUzFnd09sRG5IWkVlcW9JNXBzb25qUVo2WjVvRXdxdUt3VnZjbk5vN1hsNVpMTUNQMkUtOVR4QUc3M05NVUZKU2xzNmVn?oc=5</t>
         </is>
       </c>
       <c r="F85" t="n">
         <v>7</v>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46054.85417824074</v>
+        <v>46055.47577546296</v>
       </c>
     </row>
     <row r="86">
@@ -3242,24 +3242,24 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Tesla cuts car models in shift to robots and AI - BBC</t>
+          <t>One Identity names Gihan Munasinghe chief technology officer - IT Brief UK</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Thu, 29 Jan 2026 02:35:07 GMT</t>
+          <t>Mon, 02 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBrMFdIUU1aRzA0bVlsQ2hpQUhralNORFB4S1FfcVUwUEFaQ1o2bDV1VVA4UHhSakpIU2tmRlNjU3lWOFI1UGNkWWdYdTZJUDIxXzRYcUxXZ0tMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOcnhlcVU0RWd5WDI4R0s5d0lvQmdaVHZQeW9QblFnTV8tYmJ2UjlWY1NCckNEWmZiR1lGc19GV3k3ZmMzaF9XV0IwQXBNSEp1N0hTQkhmcW1Wa2ozVmZGUDYzSHh4bFo4UzMwc2FzMmNLTXMzRWw2Y3ZkVHRxYWo4N214NThWRUhHRzN4eHRZbTB1UQ?oc=5</t>
         </is>
       </c>
       <c r="F86" t="n">
         <v>7</v>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46051.10771990741</v>
+        <v>46055.5</v>
       </c>
     </row>
     <row r="87">
@@ -3275,24 +3275,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Tesla Recasts Identity As Robotics And AI Platform With Merger Potential - Yahoo Finance UK</t>
+          <t>Breakthrough Power Module Aims to Ease Energy Strain from AI and Data Centers - Telecom Review Africa</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 17:10:27 GMT</t>
+          <t>Mon, 02 Feb 2026 05:11:38 GMT</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOenZGbUM3RXE4U3Q5RUU5bmZoOC1MelduTGw2Nkl5dWpLZVY1UmNPWnpxQU9Pam1IWGtaYndOcUZWSGt3amdtZk1MQ2hOXzQxeFRETlRFWDd3UkxienlDSWhhTHN2c0hSblNnckdBaUg4V0JOQnlYdjU1VjliMF9aZ3gzNXpvQ3p0RVFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOQ293QzEtcl9tQWc2dlJOUG1MSWJwZm1pQXdxVnhiWHo4NEo3TU5YR1hzVXBGRXlQcFY4cDdfTjZPdXZBR3d1UDhXTkVtR1UybFotXzBPOUtDY3FkYndxbU9kODVOQ2RvcVYtM2FEeG80T2xLN1EwUVNZRTJkbzFBOXV5ZGRwRUJXcndkeUpfcDNLRnRxRWkxUHhiRjB6R0k2Zm9KRE1ENVh3TWZkcU5SYU1ja2NTZnJKOG52cndlYVdlN0REY2locnVVaHJLMnkwbXhERkROWTFFMzh3c3c?oc=5</t>
         </is>
       </c>
       <c r="F87" t="n">
         <v>7</v>
       </c>
       <c r="G87" s="1" t="n">
-        <v>46054.71559027778</v>
+        <v>46055.21641203704</v>
       </c>
     </row>
     <row r="88">
@@ -3308,24 +3308,24 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Managing the Load: AI and Cognitive Load in Education - Faculty Focus</t>
+          <t>EU Selects SUPREME Consortium to Develop The Union’s Superconducting Technology - The Quantum Insider</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 04:07:18 GMT</t>
+          <t>Mon, 02 Feb 2026 09:24:45 GMT</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNNUhwYkZCLS1OQk5FMnVLNThFcE05TGx2M1lEbld3bEdyT3dYdER5b0dwMnJZZW83YlBGRDIxYTRWRXp5eTJHRlRnZ0JwS0FzTHFRV3ZQRV9ZNGVqendFYmN0ekE2REVEblRMX0xWTGlUXzVsWGJLYXFjSkcyaEh4ZGt4SHZXQUU5bUFsWDgtelExVEV5bklDaHZTNk43RDkzNWNTcWwtOGZNYWlLTnY2SXhXNmtPNk9tMVpqWG1n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNaUNORlkxWXBCMW5YVjZIdHFFck9Yc2VhbGxWMElvaTI2RW01azg1cDBJTWlaclpXZENadEVsNXZiRnNpdUt3QjE5UkVkclByTTNEVXowa1VlTGZ0RlVIaWVIVkwzcjB6b1RVeTlkcjlWMXJrU2psMnNCbm1Fdkg0cW9faGpkVjFZNk1UVE1WejhXTjRfaHdaSUstY0k0UWZjeXNLYWJkbF9SUFRTWm9ZZTNXQ2VaQThROXlFXw?oc=5</t>
         </is>
       </c>
       <c r="F88" t="n">
         <v>7</v>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46055.17173611111</v>
+        <v>46055.3921875</v>
       </c>
     </row>
     <row r="89">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>C-suite poses greatest AI risk to businesses, not entry-level - Personnel Today</t>
+          <t>Betting blind on AI and the scientific mind - The Transmitter</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBhS2t1cTV0UkhxRmkxdkM0ZmU3eU1JUVR3WG5wY1lkMm1lNGZUZm85VDVYUEFJQnZmVGhKY0dfQkhGWjQ3bDk2bWdZSXRHM3U5ekc4LV9NNGs5MUc1R2owQWwtRlRUSlYwSXluN2VBTVZpS3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNdWJUT1lZS2tZZEVHXzlBbUJOaVl3Y2VLa3dXblRNcmxsci16YnBrWENIanhRRHFoY1k5VmkyenF6VzdXaGEtRW9WVFlwSXhtTFVHLTdLb1RGVTY0Y2dhZ3dWOHdPZDB1SWFNZnZoR0UyN05TNzQxYmx6eG9QRHROZERYX24tRVg0d0NKTm1OT1RRNU1WUTE0b21zT09UTW04?oc=5</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -3374,24 +3374,24 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Can agtech fulfill its promise? World Agri-Tech explores opportunities, challenges for the future - AgTechNavigator.com</t>
+          <t>UPS Resets Network To Favour Automation And Higher Margin Deliveries - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:06:00 GMT</t>
+          <t>Mon, 02 Feb 2026 01:06:00 GMT</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNWFFRQ2RucW80azhrWVJ4Y2J2enBFdDJHOTVlcXhnNWtDTmJsOWdadnQ0cUVHNzRXSGhlUGZweUI4RlZGWHA2cFRRRUl6YVhxNzNFYVd1d3dMMFU0LVJXbTA5Zk80ME14ZGhoVjdpVzRXUFZtV0pWb010Z2kwZWliVXV6Z0FkYlBqSmN1b3F6YklmTWxVWWtpVzh0RnhCYWZ3Qm9KLTlrUEFJUnBtdkNrVVpR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNaVo5eHdfOGZhUjJoM0RQeTBpbWNDb0NkdnZKclhQcWtCc2NJUGFmTVBZQmNwcFdibW9QY2JfVjVMTDRiMjNWRkxaU1VPd2hYOWlZSS1GUlJjWFlGMjBfVWZETUVBaUNsUENXVkJ4eDVBNVN6Y2dkNFRVSzBPQXc4dkFqZXNPR2d3QVV4SWRB?oc=5</t>
         </is>
       </c>
       <c r="F90" t="n">
         <v>7</v>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46055.42083333333</v>
+        <v>46055.04583333333</v>
       </c>
     </row>
     <row r="91">
@@ -3407,24 +3407,24 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>China, AI and the West’s Free Speech Crackdown | Ash Sarkar Meets Ai Weiwei - Novara Media</t>
+          <t>Tarabut acquires Servable to add financial AI capabilities - Retail Banker International</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 15:03:30 GMT</t>
+          <t>Mon, 02 Feb 2026 11:43:07 GMT</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQVlRxZHhhcHV0NGFidnJRcWZkQnc3WWZLQkNiR1M0T0JSZU9MaGc3VkprNWVvWkZfUVpaaHFxUVFHdkpjdUNWSWRiYno0cXhpOXZNWWF5LWJCV3NzRVJCM1lhbkc1YkFmNUg4ZG9FZ3p4RTJEZUNKeUtIVkh1cDVzTzdMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE4zbkhCOEtya20wSGRvRG1UNHkwTGN0NmlmWFNXdUMzOThtTVdaUGhDeFh0T0YtdzlDa2dCdXFHYUkzdUJjb2d5dngySGY2aWl2Vko4Z0s1dUFJbHBUeFZVRGpOR1I3SHVMLTREeUJnS0VDR2NUTXpLbm9BdXBJZw?oc=5</t>
         </is>
       </c>
       <c r="F91" t="n">
         <v>7</v>
       </c>
       <c r="G91" s="1" t="n">
-        <v>46054.62743055556</v>
+        <v>46055.48827546297</v>
       </c>
     </row>
     <row r="92">
@@ -3440,24 +3440,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Why are women more sceptical of AI than men? New study sheds light - Euronews.com</t>
+          <t>Tesla cuts car models in shift to robots and AI - BBC</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:30:46 GMT</t>
+          <t>Thu, 29 Jan 2026 02:35:07 GMT</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPd285WTNKeFhFUUFjOW1qekVOX1dVeFBuZ1I4aGtZdjhsMFcwck00SGdRdHFkRmk5ZTM1Xzd1MDFtVkZYX29qRVR4RFY0Z21NTDhBRmhaZmV2azI5Uy1oTW9VbDRUS2thS0RYQWtLZDFIXzFiMGNNVjc3LXJNRk5CcTEzalNFQjNPUU1hbmRfcGJlRzZEd2I3c0FBMHFHVWltRDV3aHJBSnRZdWhPbVBfVmhKQVluQ1VCT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBrMFdIUU1aRzA0bVlsQ2hpQUhralNORFB4S1FfcVUwUEFaQ1o2bDV1VVA4UHhSakpIU2tmRlNjU3lWOFI1UGNkWWdYdTZJUDIxXzRYcUxXZ0tMQQ?oc=5</t>
         </is>
       </c>
       <c r="F92" t="n">
         <v>7</v>
       </c>
       <c r="G92" s="1" t="n">
-        <v>46055.35469907407</v>
+        <v>46051.10771990741</v>
       </c>
     </row>
     <row r="93">
@@ -3473,24 +3473,24 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>AI’s ongoing evolution in corporate travel - PhocusWire</t>
+          <t>Microsoft Q2 2026 Earnings: Can AI and Cloud Keep CX Ahead of the Curve? - CX Today</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:04:25 GMT</t>
+          <t>Mon, 02 Feb 2026 10:46:47 GMT</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQNnRpVmpSMDE0TWZYaXlNalhkMHN6VzdTWGJtbGtXdnd4bUhzZWpQS3dDUFVZaDdteGJxNGUySnBwMkJuemQ0U1ZVVF9XX2U2bktCa3BxcFdKQjBIOVZiUlhldm52YWNBOWpneWpQQWZXMlZvOFRiYXVJTTAxVndtdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNUC1EZDJEcjROV0lVNzhneHVKWXk5NEcxZHk3OVZ5ellocGZJUnpTbHI2ZmNBbDVYY19SbS1XWGotdC1ISzE1S3RiT3dqWEFBY0JpUzlndDRCRlJ5SmdfZ2JhSlZQMUJsLUQ5UHA4NGZ3dlVKYmlRbnN6akZKSWZMbWxPWGtOOEVfZ24tMHBNMmZCam5ZeFhlRkkxd001SS1qanpXanNWM2xQQjNVaTRaV2Rvb0hLQQ?oc=5</t>
         </is>
       </c>
       <c r="F93" t="n">
         <v>7</v>
       </c>
       <c r="G93" s="1" t="n">
-        <v>46055.25306712963</v>
+        <v>46055.4491550926</v>
       </c>
     </row>
     <row r="94">
@@ -3506,24 +3506,24 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Deezer opens AI detection tool to rivals - Digital Watch Observatory</t>
+          <t>Maxio Report suggests B2B SaaS and AI growth remains strong but has become more selective - Enterprise Times</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:05:00 GMT</t>
+          <t>Mon, 02 Feb 2026 07:14:23 GMT</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9ackFocUVZY1ltM2ZxaVpSQWFCcmdGTGVmRkN4WW10LXZJZlVFckQzQnc5RElZWmNvbzhPTEZVbFFLOGdwNm5RcE5ncmt3UkxoUXRRVzluTnlRMndvcXNYNmVQY01XOFpZeVlzck4tSF9TZTIy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxQS1Y4c09NU1JsSUlBMjFudjlEUGlkX19mdWR6Wm5pZ3VpV0NMd0JFTjY4YmtPd1VqWjRzb2E3aGNyMjlxSlBUVm5aMnl5Z1RabC1rNEZpcW1mSURYaUZVVko5dUNkQ2kzekltTDR4dHpTQS1uZFFHN2hWYS0zYnl1NEp5UERRczJwU2pKUnkzakN3c3RZaXM2R3EwX0tXZWgxcUlVRmRwOTc4OGxacmRWbjM3WXNQaUNYcnhwOXptTXpHU2RpRWpNaVEwUEU1UzZR?oc=5</t>
         </is>
       </c>
       <c r="F94" t="n">
         <v>7</v>
       </c>
       <c r="G94" s="1" t="n">
-        <v>46055.33680555555</v>
+        <v>46055.30165509259</v>
       </c>
     </row>
     <row r="95">
@@ -3539,24 +3539,24 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>PE-backed iamproperty swoops for lead gen firm - businesscloud.co.uk</t>
+          <t>CANSO Says Greater Airspace Capacity Requires Automation and Strategy - Aviation Week Network</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:49:22 GMT</t>
+          <t>Mon, 02 Feb 2026 12:39:01 GMT</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPdzRvT2ZVbUFmYS1tbXNnNEVwbVVNUEJiSnczTmhYOTRaLUdpWUhwV3ZiczNYcl9nZ3VWbW1YZkkyR3BlVENSdDBRbmNuT3B6My1BdjU2R3ltbFFJNkUtTWN4OXJSd3F6Vk9QVFlCU2cyMGZQUXZJYS1DUGhJdDlidFFwdWNXVjQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQeEpFajRYUjU3cDhISm9odXVmaF9BU01aZFZxNndTd3AyUnJyZWV1MVdsbjQ5SEt4UlZ4LTJTTFkxdW9lR0xITzY2TFpWQmJiRDhYTzNyQnJhWDNhY3g3bTQwdHVXd3J5ekFtdnlJZ3M4ODU0NWE0VFllMHRBTEpUbTh5OWJBT3cwcllYWHdlZ00yUFNOX3lSNGtKZk40aXpBVzNSVllCeUFmeDkwaVdSM1pFMTZsbEp5SFkwOFpfbw?oc=5</t>
         </is>
       </c>
       <c r="F95" t="n">
         <v>7</v>
       </c>
       <c r="G95" s="1" t="n">
-        <v>46055.28428240741</v>
+        <v>46055.5270949074</v>
       </c>
     </row>
     <row r="96">
@@ -3572,24 +3572,24 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>KPMG warns of gaps between AI ambition and returns - Digital Watch Observatory</t>
+          <t>Why are women more sceptical of AI than men? New study sheds light - Euronews.com</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 08:30:46 GMT</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPa0NUQkc4cm94QjhSZ1ppc1Bmb19FUW9RTGNjWDdGUHJncnFpeXNFdkJYS09LTHk2dGRQVUkzb2ZyMGxYOVJyeXlXSzJyMGwyTkdQOVpjX2NDVHMwalNMTkpoWTdPbm1NR1dRRDNKQ1pGbnBBZ1pzOVlRalJCM3dDQ1p3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPd285WTNKeFhFUUFjOW1qekVOX1dVeFBuZ1I4aGtZdjhsMFcwck00SGdRdHFkRmk5ZTM1Xzd1MDFtVkZYX29qRVR4RFY0Z21NTDhBRmhaZmV2azI5Uy1oTW9VbDRUS2thS0RYQWtLZDFIXzFiMGNNVjc3LXJNRk5CcTEzalNFQjNPUU1hbmRfcGJlRzZEd2I3c0FBMHFHVWltRDV3aHJBSnRZdWhPbVBfVmhKQVluQ1VCT1E?oc=5</t>
         </is>
       </c>
       <c r="F96" t="n">
         <v>7</v>
       </c>
       <c r="G96" s="1" t="n">
-        <v>46055.375</v>
+        <v>46055.35469907407</v>
       </c>
     </row>
     <row r="97">
@@ -3605,24 +3605,24 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Venture Investment in AI Rises Fivefold in Two Years, Says Latest Report - The Astana Times</t>
+          <t>Grok, AI and “free speech” – Starmer vs Musk - palatinate.org.uk</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 04:52:40 GMT</t>
+          <t>Sun, 01 Feb 2026 20:30:01 GMT</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPVHdSRUZ1LTFkVDJ0VE9td2pIY0xHaThneU82YXFyN2Ric2JQSWpjTHY4WjR5ZDlDbXVMZHpVbTRvLWlTQnl3WlZYYTltYjh2ZGJuYTRkbkNoa0N6ZFV2MEU2RVNNZ0x6b3NoU1ZvdGRiX3QyVmpPNG0wREpJVEZ3VmZ1QS1VRWI3NWN6UXg1em96UTVkdjJVUTZSOXl1ZFF2MHE0ZTFwVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE9Qa2J6bG5BUjIzZ2k0Zkl6Ynk4a0x3dl9Hbm1yenJMNE1iUFM1cVY4d0hUcmdwYk5XRTB5a3ZjN0h6eldTVU41TkdWV185ZzFLQ0VCZkdkVU9keFZubF9kV0ZsQUdteE5jdDlKdHRpdUdjNXRacVpwMDR3?oc=5</t>
         </is>
       </c>
       <c r="F97" t="n">
         <v>7</v>
       </c>
       <c r="G97" s="1" t="n">
-        <v>46055.20324074074</v>
+        <v>46054.85417824074</v>
       </c>
     </row>
     <row r="98">
@@ -3638,24 +3638,24 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>AI in court cases and court cases about AI: eight legal tech stories that you might have missed - The Law Society</t>
+          <t>Can agtech fulfill its promise? World Agri-Tech explores opportunities, challenges for the future - AgTechNavigator.com</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 14:28:45 GMT</t>
+          <t>Mon, 02 Feb 2026 10:06:00 GMT</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNdUJSVzJudnlnMlUxOFphSmQyNmoxenBwSnhrWHF1WEc3S2FUSF80R2hGRjRIUWZIaXhkLXBRY0Y4dy1DWC1KM053Smk2dEhqOTc0X1dMY3hCbGhpdmsxR2xZT0tLdVlYejBmcExCZHJxcVRLbWpkWUJjOWctSTI4VWsyNFotb0ZrQS1TM1RURG9HcFpWd3I5UUhWdXRsMFhodWpER1RNVUxhWU5IWEVnaWtvNEVWb1RTQlJHX0RSbFRHdmt4UkF1Q2dxMEQ3SFJUQUVKQW9WcnRpUWtXU3Z0RFpKZlNEOFU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNWFFRQ2RucW80azhrWVJ4Y2J2enBFdDJHOTVlcXhnNWtDTmJsOWdadnQ0cUVHNzRXSGhlUGZweUI4RlZGWHA2cFRRRUl6YVhxNzNFYVd1d3dMMFU0LVJXbTA5Zk80ME14ZGhoVjdpVzRXUFZtV0pWb010Z2kwZWliVXV6Z0FkYlBqSmN1b3F6YklmTWxVWWtpVzh0RnhCYWZ3Qm9KLTlrUEFJUnBtdkNrVVpR?oc=5</t>
         </is>
       </c>
       <c r="F98" t="n">
         <v>7</v>
       </c>
       <c r="G98" s="1" t="n">
-        <v>46052.60329861111</v>
+        <v>46055.42083333333</v>
       </c>
     </row>
     <row r="99">
@@ -3671,24 +3671,24 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Starbucks bets on robots to brew a turnaround in customers - BBC</t>
+          <t>Tesla Recasts Identity As Robotics And AI Platform With Merger Potential - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 00:11:06 GMT</t>
+          <t>Sun, 01 Feb 2026 17:10:27 GMT</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5nSFI2ZTA2QTdDc3FqelRieW9rT0N4OXU1Mmc3YmtLd2V0Si04SmtQdlVqOG50ZEJKR1NnXzA5YmVjQUk0elRaeXZuZi15cl9zYTV0VUFRc1pMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOenZGbUM3RXE4U3Q5RUU5bmZoOC1MelduTGw2Nkl5dWpLZVY1UmNPWnpxQU9Pam1IWGtaYndOcUZWSGt3amdtZk1MQ2hOXzQxeFRETlRFWDd3UkxienlDSWhhTHN2c0hSblNnckdBaUg4V0JOQnlYdjU1VjliMF9aZ3gzNXpvQ3p0RVFR?oc=5</t>
         </is>
       </c>
       <c r="F99" t="n">
         <v>7</v>
       </c>
       <c r="G99" s="1" t="n">
-        <v>46055.00770833333</v>
+        <v>46054.71559027778</v>
       </c>
     </row>
     <row r="100">
@@ -3704,24 +3704,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Who Answers When We Ask AI About God? - EWTN Vatican</t>
+          <t>Managing the Load: AI and Cognitive Load in Education - Faculty Focus</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:26:40 GMT</t>
+          <t>Mon, 02 Feb 2026 04:07:18 GMT</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFB5NklNUjczbU81ZU1UdzdnaGdKak80OFJseVEyX2hKbUY2VVN4VUJBSGtBcUo2NGtTYkIxMDVsUHE0TlRfNlI1ekRScDExMjNDbHdUeVpVbkI4TTBPV3Z2NHpoakN5OVB0LWgzVlBlS0txeGJIN2RqemZfVmlkdDg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNNUhwYkZCLS1OQk5FMnVLNThFcE05TGx2M1lEbld3bEdyT3dYdER5b0dwMnJZZW83YlBGRDIxYTRWRXp5eTJHRlRnZ0JwS0FzTHFRV3ZQRV9ZNGVqendFYmN0ekE2REVEblRMX0xWTGlUXzVsWGJLYXFjSkcyaEh4ZGt4SHZXQUU5bUFsWDgtelExVEV5bklDaHZTNk43RDkzNWNTcWwtOGZNYWlLTnY2SXhXNmtPNk9tMVpqWG1n?oc=5</t>
         </is>
       </c>
       <c r="F100" t="n">
         <v>7</v>
       </c>
       <c r="G100" s="1" t="n">
-        <v>46055.35185185185</v>
+        <v>46055.17173611111</v>
       </c>
     </row>
     <row r="101">
@@ -3737,24 +3737,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CyberCatch Announces Acquisition of Multi-Authority Attributes-Based Encryption, Expands Product Offering to Boost Cybersecurity, Mitigate Risk From AI and Quantum Driven Cyber Attacks and Drive Large Cybersecurity Sales - Yahoo Finance</t>
+          <t>C-suite poses greatest AI risk to businesses, not entry-level - Personnel Today</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 05:00:58 GMT</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQaHlQc3pwZUdRUjF2VGtEN1RoMlJCbnpHTFJFVU03bVg0Y2RBbXJXTHZVMmFtdjFwQW9KVklDYlhORUxBeVRXZlZISmFadmotY2pLZlFBMUEwc1kyQnlhMkVhRUdLNGJIUmlxc0JBdWFmWVJCZ3JxSWU4akdGQWtxTWlLZ2dJb3Q4V2Iza0gwT2dORkRKYnR3RTdR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBhS2t1cTV0UkhxRmkxdkM0ZmU3eU1JUVR3WG5wY1lkMm1lNGZUZm85VDVYUEFJQnZmVGhKY0dfQkhGWjQ3bDk2bWdZSXRHM3U5ekc4LV9NNGs5MUc1R2owQWwtRlRUSlYwSXluN2VBTVZpS3M?oc=5</t>
         </is>
       </c>
       <c r="F101" t="n">
         <v>7</v>
       </c>
       <c r="G101" s="1" t="n">
-        <v>46055.41666666666</v>
+        <v>46055.20900462963</v>
       </c>
     </row>
     <row r="102">
@@ -3770,24 +3770,24 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Can workers compete with machines and stay relevant in the AI era? - UN News</t>
+          <t>AI’s ongoing evolution in corporate travel - PhocusWire</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 05:01:00 GMT</t>
+          <t>Mon, 02 Feb 2026 06:04:25 GMT</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTFBNMHZBbWdCSDdBX19fY1ptWTlza1NsY25LWWNlalk2UEhoQUVrVUE5ekNhQURiMC1KTGJXSldPRUp3SFUta0lzazdoNEVCVGhFVHFmU0JTZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQNnRpVmpSMDE0TWZYaXlNalhkMHN6VzdTWGJtbGtXdnd4bUhzZWpQS3dDUFVZaDdteGJxNGUySnBwMkJuemQ0U1ZVVF9XX2U2bktCa3BxcFdKQjBIOVZiUlhldm52YWNBOWpneWpQQWZXMlZvOFRiYXVJTTAxVndtdA?oc=5</t>
         </is>
       </c>
       <c r="F102" t="n">
         <v>7</v>
       </c>
       <c r="G102" s="1" t="n">
-        <v>46053.20902777778</v>
+        <v>46055.25306712963</v>
       </c>
     </row>
     <row r="103">
@@ -3803,24 +3803,24 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>How technology can help bank Africa’s informal economy - The World Economic Forum</t>
+          <t>Deezer opens AI detection tool to rivals - Digital Watch Observatory</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 08:05:00 GMT</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQY2VyZW5aLWxNNlhIajNPWXJfN0ZCSXh2T0xWSTdpX01yeUxoMGYxVl9tQ0xZdXhZMWJnX3JYMHg3YUkwZXdDdHJRTlNGLWtDM2doendjWTJKZVNmZjFxejlSbEYtalVKX0o0MVVUYjJIZVhNMkZFelIxem5DXzhzemZ2b0QtcHY2ckxrZG0zQ3ZLSnAzbkozOXhkZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9ackFocUVZY1ltM2ZxaVpSQWFCcmdGTGVmRkN4WW10LXZJZlVFckQzQnc5RElZWmNvbzhPTEZVbFFLOGdwNm5RcE5ncmt3UkxoUXRRVzluTnlRMndvcXNYNmVQY01XOFpZeVlzck4tSF9TZTIy?oc=5</t>
         </is>
       </c>
       <c r="F103" t="n">
         <v>7</v>
       </c>
       <c r="G103" s="1" t="n">
-        <v>46055.33333333334</v>
+        <v>46055.33680555555</v>
       </c>
     </row>
     <row r="104">
@@ -3836,24 +3836,24 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Opinion | Where Is A.I. Taking Us? Eight Leading Thinkers Share Their Visions. - The New York Times</t>
+          <t>China, AI and the West’s Free Speech Crackdown | Ash Sarkar Meets Ai Weiwei - Novara Media</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:03:00 GMT</t>
+          <t>Sun, 01 Feb 2026 15:03:30 GMT</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPXy1tbFc5V2p0NVlhcHJUc2FQeFZkS21UMjQ5NXdkcUZib2VndHZOenBpTW5uOGZvYTRoUUZSN2tZT1c3M19XbDEtbkpVY1pPbWJmdmp5RDZuVFZtWDkyb0ZhbExleXl1NnBCVTJWSktzRHhicldUMnFOSmpLOXdLck5waWpnTUktenh4WmRsZExTdkNELXFwVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQVlRxZHhhcHV0NGFidnJRcWZkQnc3WWZLQkNiR1M0T0JSZU9MaGc3VkprNWVvWkZfUVpaaHFxUVFHdkpjdUNWSWRiYno0cXhpOXZNWWF5LWJCV3NzRVJCM1lhbkc1YkFmNUg4ZG9FZ3p4RTJEZUNKeUtIVkh1cDVzTzdMQQ?oc=5</t>
         </is>
       </c>
       <c r="F104" t="n">
         <v>7</v>
       </c>
       <c r="G104" s="1" t="n">
-        <v>46055.41875</v>
+        <v>46054.62743055556</v>
       </c>
     </row>
     <row r="105">
@@ -3869,24 +3869,24 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>West Midlands AI and coding trainer to open new Dubai base - BBC</t>
+          <t>Kazakhstan to Introduce AI in Water Sector by May, PM Bektenov Says - The Astana Times</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Wed, 28 Jan 2026 06:05:45 GMT</t>
+          <t>Mon, 02 Feb 2026 12:37:49 GMT</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1XN1BWU1ZLb24yclpFYnFDdmJwcHVXclBCb3EzLW1TZnRVUUE4OHpldEFPTFlobUpjdjBHM0NuakdnMEJyR2oxMjBHZFJPekFNU0tpVXNuMm9QUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNT2JBTHhOTmhnTTBtcWQ5NTVCR05aeW5oZnlxNTlyQzVYbllIWHdXX010Y3R5amFnUEN6U3d6Q1R4NVZZMnVhUVJiM3pmWVUyRzl3UTh4WUhwQjV4LUlRZ0k2TmlzUWx5QkhWdl9UbTNvUmRwNUM2VE91a3dCZEpmQlBqMVdSSlNpdnF1RHZKcTZ2UjRBcmRiWjR2ZWV2TFdu?oc=5</t>
         </is>
       </c>
       <c r="F105" t="n">
         <v>7</v>
       </c>
       <c r="G105" s="1" t="n">
-        <v>46050.25399305556</v>
+        <v>46055.52626157407</v>
       </c>
     </row>
     <row r="106">
@@ -3902,24 +3902,24 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Did artificial intelligence really drive layoffs at Amazon and other firms? It can be hard to tell - ABC News</t>
+          <t>AI in court cases and court cases about AI: eight legal tech stories that you might have missed - The Law Society</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:56:30 GMT</t>
+          <t>Fri, 30 Jan 2026 14:28:45 GMT</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQVlZsdjAwQnBlUFo1c3ZlZDBudDRoVnB1SzZ6c2oyTG9aZXZtVkY4bkI0aEczN3hFbUF3UmxXV3I0TzZPaEtkRk1BbUljel9HYlRPR0RHdEt4UVY1WXJZS3NMdFotb2MzZlVpakpWTWdtLW90MGNVdGh2ejZDLS1VaGNxRm4tbGJKT1JhTThjdXhHLXhLVFMxNWdxTUcwcGx5cEpDNUtXaHFZWE3SAbABQVVfeXFMT1RmcVhCUi1sVnBfeXNOM1k5ZUVPWWJndEdEcThMT1JTdktFRWJ0U0JreUFhT3o5S0plWl8xQ1dTUE1vbkU1Q2QwcDQ3bmJfbDZFZWs0UzNfUEFJOVlNLS1uM3ZUREdLcE1Cb010c3JuMmdySEZaNENzQ0xtYjJKX05CRmhuZGRjSHBuWklVUVh2YVc0QzhZd1Q0X3FlNUxhVk10bTVtbnpzeGNfYjl5YmM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNdUJSVzJudnlnMlUxOFphSmQyNmoxenBwSnhrWHF1WEc3S2FUSF80R2hGRjRIUWZIaXhkLXBRY0Y4dy1DWC1KM053Smk2dEhqOTc0X1dMY3hCbGhpdmsxR2xZT0tLdVlYejBmcExCZHJxcVRLbWpkWUJjOWctSTI4VWsyNFotb0ZrQS1TM1RURG9HcFpWd3I5UUhWdXRsMFhodWpER1RNVUxhWU5IWEVnaWtvNEVWb1RTQlJHX0RSbFRHdmt4UkF1Q2dxMEQ3SFJUQUVKQW9WcnRpUWtXU3Z0RFpKZlNEOFU?oc=5</t>
         </is>
       </c>
       <c r="F106" t="n">
         <v>7</v>
       </c>
       <c r="G106" s="1" t="n">
-        <v>46055.37256944444</v>
+        <v>46052.60329861111</v>
       </c>
     </row>
     <row r="107">
@@ -3935,24 +3935,24 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Leading with AI: How communicators can build authentic leadership at scale - PR Daily</t>
+          <t>KPMG warns of gaps between AI ambition and returns - Digital Watch Observatory</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:01:06 GMT</t>
+          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQTDVCZERTUTl5N0hLckZyR3lCbkNvdTF4eEJaTU5aTTJiWm1FbHpXOHE0dmdBR2FZZWh3Mi1obU8tLWgzRkNmeS0yQ0gzbGJWM2JlX1FwTkF6ZkN1V1I1NUNKaXBJb182TlI3MnRqVlRQZEREMTBXSjFFS3hxNzM5emFpWnRTb0R4ZGNqNHVfWk4xNUQ3ZXlRbEVKcmdaTUk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPa0NUQkc4cm94QjhSZ1ppc1Bmb19FUW9RTGNjWDdGUHJncnFpeXNFdkJYS09LTHk2dGRQVUkzb2ZyMGxYOVJyeXlXSzJyMGwyTkdQOVpjX2NDVHMwalNMTkpoWTdPbm1NR1dRRDNKQ1pGbnBBZ1pzOVlRalJCM3dDQ1p3?oc=5</t>
         </is>
       </c>
       <c r="F107" t="n">
         <v>7</v>
       </c>
       <c r="G107" s="1" t="n">
-        <v>46055.37576388889</v>
+        <v>46055.375</v>
       </c>
     </row>
     <row r="108">
@@ -3968,24 +3968,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Meta's Mark Zuckerberg Just Predicted What's Next for AI (And It's Excellent News for Nvidia) - The Motley Fool</t>
+          <t>Venture Investment in AI Rises Fivefold in Two Years, Says Latest Report - The Astana Times</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 23:45:00 GMT</t>
+          <t>Mon, 02 Feb 2026 04:52:40 GMT</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQSTRyeUlndVlXLTMwZzVIdldoc0dJWTNLQlF5Q3hfZm5Ia2NLRkduYUUxcEI1MHl0LVpGa2ZGajFLTlNuak1Na0hMMTFTZktmbWtUY3kzeGRHRDN1M0ZIMnZfX2p3MUZzbzFkY3lSZGg1b1ZrRFJXbGR3cngtcTJtU2VkUDdFaVdnNTdXMUhRdkY0aWlOcUpfVg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPVHdSRUZ1LTFkVDJ0VE9td2pIY0xHaThneU82YXFyN2Ric2JQSWpjTHY4WjR5ZDlDbXVMZHpVbTRvLWlTQnl3WlZYYTltYjh2ZGJuYTRkbkNoa0N6ZFV2MEU2RVNNZ0x6b3NoU1ZvdGRiX3QyVmpPNG0wREpJVEZ3VmZ1QS1VRWI3NWN6UXg1em96UTVkdjJVUTZSOXl1ZFF2MHE0ZTFwVQ?oc=5</t>
         </is>
       </c>
       <c r="F108" t="n">
         <v>7</v>
       </c>
       <c r="G108" s="1" t="n">
-        <v>46054.98958333334</v>
+        <v>46055.20324074074</v>
       </c>
     </row>
     <row r="109">
@@ -4001,24 +4001,24 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Japan, Britain to boost cybersecurity and critical minerals cooperation as China’s influence grows - ABC News</t>
+          <t>Starbucks bets on robots to brew a turnaround and win customers - BBC</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Sat, 31 Jan 2026 15:07:22 GMT</t>
+          <t>Mon, 02 Feb 2026 00:11:06 GMT</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNSGRIVS1GM1BIeGhYUUo4Q2QxeHNINFQzR2NMR0hhbDNRX0xOeGtuSjV5YjRMbmVvdEN2dXpzREx3Uk9nNWJSZzZkZFBJTk9xbHJBZ0pfVS16M1ZWajZQUjVzaEltb1M3Wi1RZElqWjYwLTFCTzAzVExybVRIRXEtUDRTdWlsSXpOVUJiQkVnQnBTLU1sQXZDRjB3Rlp3V0lqR2RndGU5Uk9aVVhkcjJtMGw1eldtWjRoeFJqM2xUZjlBSkhpWVHSAcsBQVVfeXFMTWhiN3lYSjdEOS0tdkpIbE1OU1VfclRyQzlYWlF6VTQ4cmhleHQ0OWtxYzZJQ1pfbVlOYUhVQ09oUUo5RFJsWFRZTWVsY24wS1JLMmFGbVd3cGxHZUNvdnVkU200Q2VvMXVmMTR2cFFWS3pyVlNyWldTalZ5MXBrNTZ1eGMzMTFGT1NZNzBWYWtfQldvZjFkRThUb0UtUGF1WTBiSjdGVFQ2TGdvOWRQbkdxNFQ0VmtpZVd4YThvWXRCb1pUc04tU084LVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5nSFI2ZTA2QTdDc3FqelRieW9rT0N4OXU1Mmc3YmtLd2V0Si04SmtQdlVqOG50ZEJKR1NnXzA5YmVjQUk0elRaeXZuZi15cl9zYTV0VUFRc1pMQQ?oc=5</t>
         </is>
       </c>
       <c r="F109" t="n">
         <v>7</v>
       </c>
       <c r="G109" s="1" t="n">
-        <v>46053.63011574074</v>
+        <v>46055.00770833333</v>
       </c>
     </row>
     <row r="110">
@@ -4034,24 +4034,24 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Tesla energy storage deployments jumped in ‘crucial AI transformation year'; company expects margin compression in 2026 - Energy-Storage.News</t>
+          <t>Who Answers When We Ask AI About God? - EWTN Vatican</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:27:08 GMT</t>
+          <t>Mon, 02 Feb 2026 08:26:40 GMT</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNX2dkTDM3VzFxQ0F1RFhVRE5vRzlLTWg0aVYzalVqaVZCckVqdF9HeW5VM0duOVozbG90Y2VqMk4ybGlBNTlGY0lqckJUTDJXZXgzZUhBNWpYRFhMOGc1eTBuLUM0QkJ5bXdHazVmM2xVck1wNFpuRllWUGt3aG9jcFRVcDdPZmlZZ2U2d24tY0I0MTh6WmFUcWUtdUhvZDF4NVltbXcyUlgyTy1Dem1pWVBTbDljOUdTamM5MUVPaDZfblAzWDN3VGNQU3FnNWdObk9YcTlvWGtsTWtIYmR6RHJzRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFB5NklNUjczbU81ZU1UdzdnaGdKak80OFJseVEyX2hKbUY2VVN4VUJBSGtBcUo2NGtTYkIxMDVsUHE0TlRfNlI1ekRScDExMjNDbHdUeVpVbkI4TTBPV3Z2NHpoakN5OVB0LWgzVlBlS0txeGJIN2RqemZfVmlkdDg?oc=5</t>
         </is>
       </c>
       <c r="F110" t="n">
         <v>7</v>
       </c>
       <c r="G110" s="1" t="n">
-        <v>46055.3938425926</v>
+        <v>46055.35185185185</v>
       </c>
     </row>
     <row r="111">
@@ -4067,24 +4067,24 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>India courts Big Tech with long‑term tax breaks as it doubles down on AI ambitions - CNBC</t>
+          <t>Opinion | Where Is A.I. Taking Us? Eight Leading Thinkers Share Their Visions. - The New York Times</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:37:50 GMT</t>
+          <t>Mon, 02 Feb 2026 10:03:00 GMT</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9JalQzUkFrUjkzT2k3UlVTcVFPelhxaFNEY0puRVBCbnY2SDc3cEJwZTktS3VFZVRrMFlzR1VkSUg3cHNvRVhnMFAtdE1qcWFuUGxKVE9paWVBRnB3T093SmdkdnRHNm9BeWw3QVNiMXc3TnRPc0hNZENRTndxd9IBgwFBVV95cUxNUmhXbmF1QnI2cEhLdGxSVW1jWGdSY2NRckVodzUyWE5MWUl4ZDFSeENwTmI4Ny1lM0Y5WWZzcDBUd2hOV1FDSVNqaVlHWG43Y09xSzZGLTBLSTBqelgxdEJqOS1Fa2Q0NWFGZU1lTlpNaVNBVlVwdWV6VERObDJWdDY0cw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPXy1tbFc5V2p0NVlhcHJUc2FQeFZkS21UMjQ5NXdkcUZib2VndHZOenBpTW5uOGZvYTRoUUZSN2tZT1c3M19XbDEtbkpVY1pPbWJmdmp5RDZuVFZtWDkyb0ZhbExleXl1NnBCVTJWSktzRHhicldUMnFOSmpLOXdLck5waWpnTUktenh4WmRsZExTdkNELXFwVQ?oc=5</t>
         </is>
       </c>
       <c r="F111" t="n">
         <v>7</v>
       </c>
       <c r="G111" s="1" t="n">
-        <v>46055.35960648148</v>
+        <v>46055.41875</v>
       </c>
     </row>
     <row r="112">
@@ -4100,24 +4100,24 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>How AI Is Changing the Storied McKinsey Interview - Business Insider</t>
+          <t>How AI is Revolutionizing Life-Saving Drug Discovery - Pharmaceutical Executive</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:31:00 GMT</t>
+          <t>Mon, 02 Feb 2026 11:06:40 GMT</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPTGQyZlRzS3c2MDdEQ1JKaWIzYlFkOHZEY1JKZWx2bkRfRTBLQW9mTGM5ZWk2dmFXQnpVcHA2dEJ3QTBQRkVRQnVJMjhSejFKdTBXbHh3VGlRSGMtcEh1S0hhNnktem5VLWZFTEJGdUI5SXpDUTBHdEF3a0NoUVhSMXJyMk5ac1U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOZlkyRDlhc3RUM0EteE5ObTBkSE9IUmZGMzBjX3VYYmZ3bW9oN0x5aWRFYWZfMTdpRmNMZGxYYmNLZjhLZEZLNlNRck8tdXR3X3Y5T3BDV0hubWwwMlE4NFV2Tm9OM0wtcUowUDdpcG5aUVF0TW53QkQ5M1BZLUJVVjJrbEo?oc=5</t>
         </is>
       </c>
       <c r="F112" t="n">
         <v>7</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>46055.43819444445</v>
+        <v>46055.46296296296</v>
       </c>
     </row>
     <row r="113">
@@ -4133,24 +4133,24 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>AI and digital skills seen as key for persons with disabilities - Digital Watch Observatory</t>
+          <t>Is AI killing productivity? - InfoWorld</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 09:00:41 GMT</t>
+          <t>Mon, 02 Feb 2026 09:04:02 GMT</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE5BWlNGWXRkZFJuUGNyMVMwQlVaZUVpRWpmU1hCaXhpbGFYWTRjTHRfcHBHcnNLTlI1WUFDQVBDSkhkeTk3MG5XUzkyWW1hbFhfSWZVVTllUlg4QmRERXdoazBzdUY2czVuRDh4UlktWFVnVmREdm54dUNaVFQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTFB1VTZOQWpQSWhQbjRZQWZyS0pCbkxuWi1EVHhQSWtKV0RmSTAyeENSVGVrcklaZnJLTUxuaGVBSHJwTnYtWXU5VVlFcGJPVC1qdWQzNzRsUXJram1GdHJCQzVHalV0ZFhZd1ptaWhabUtrd1RoRlNVUFoxZ1V2dw?oc=5</t>
         </is>
       </c>
       <c r="F113" t="n">
         <v>7</v>
       </c>
       <c r="G113" s="1" t="n">
-        <v>46054.37547453704</v>
+        <v>46055.37780092593</v>
       </c>
     </row>
     <row r="114">
@@ -4166,155 +4166,320 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Gloucestershire Council targets AI for growth - The Forester</t>
+          <t>How technology can help bank Africa’s informal economy - The World Economic Forum</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 18:05:23 GMT</t>
+          <t>Mon, 02 Feb 2026 08:00:00 GMT</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQbU94c2I1NTRMR0VPeVh5ZWNIdElDbHhxYUNCNjRtUGJDNGdIUVF5MDZFVW1tclA5Nmhfc0F0WDNma01DS0IxRDFRU3FDcS1Id2tIM2xKcjJ1UkpwcjJxc0tXNmctRnVnV0lNNXdHUmZydWZtLVJLMUxpSnhzWVJvX0ZRMTV1dVE0UGViRG5jWUYtN1BINy1IZUo1cTR5WlJ2bVZ4TkVZc0E5aXB6Z1oyeQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQY2VyZW5aLWxNNlhIajNPWXJfN0ZCSXh2T0xWSTdpX01yeUxoMGYxVl9tQ0xZdXhZMWJnX3JYMHg3YUkwZXdDdHJRTlNGLWtDM2doendjWTJKZVNmZjFxejlSbEYtalVKX0o0MVVUYjJIZVhNMkZFelIxem5DXzhzemZ2b0QtcHY2ckxrZG0zQ3ZLSnAzbkozOXhkZw?oc=5</t>
         </is>
       </c>
       <c r="F114" t="n">
         <v>7</v>
       </c>
       <c r="G114" s="1" t="n">
-        <v>46054.75373842593</v>
+        <v>46055.33333333334</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Fraud_Scam</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Jersey businesses urged to beware of scam financial emails - BBC</t>
+          <t>West Midlands AI and coding trainer to open new Dubai base - BBC</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Tue, 27 Jan 2026 16:43:45 GMT</t>
+          <t>Wed, 28 Jan 2026 06:05:45 GMT</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1pWER4ajJRcUk3NHRXN0pMZkxGbWd4WjYzbnRzQUd2ZkwxNllfMXlFRElwSGpBSEJweHA1eXU0YnRlQldLcWFYdWU5NEFnNGNBcFF4X3RFOERzZ9IBX0FVX3lxTE1QckxlMlhjejd6enltLUl5ZzkyZ1VjeUlwcTJydUNqLUpGRVdVTTZXSkI0d1h0eUVNbS1KR3JHa3dVaVdyby0xWGVaWFJWVWwzRjFXYWwyMWxCTUlwSUxB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1XN1BWU1ZLb24yclpFYnFDdmJwcHVXclBCb3EzLW1TZnRVUUE4OHpldEFPTFlobUpjdjBHM0NuakdnMEJyR2oxMjBHZFJPekFNU0tpVXNuMm9QUQ?oc=5</t>
         </is>
       </c>
       <c r="F115" t="n">
         <v>7</v>
       </c>
       <c r="G115" s="1" t="n">
-        <v>46049.69704861111</v>
+        <v>46050.25399305556</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Fraud_Scam</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Email scams go QR - Insurance Business</t>
+          <t>Did artificial intelligence really drive layoffs at Amazon and other firms? It can be hard to tell - ABC News</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Fri, 30 Jan 2026 16:40:04 GMT</t>
+          <t>Mon, 02 Feb 2026 08:27:13 GMT</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQc2dSdFZPUVZpU29DWG42eFg3S21MdWZMNFdZY2p2cG1ha24tNmh1eWVkZk5Rc0tLYXN4SU1ORmg5WmRjbzQwaHJtMVVxM0gwb1FldUZScHJfXzVkbEp0bS02bkJERnRXMkhWOWxLcWEyYUhFUVJvQ0ZjSTY4MmRhbXVnODNMdmM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOUnd4UzhaZlNjTEVyRDVIbVgtMFJJcExLR1psMVdtWUxYcktJX05BUkFISUJLdW11Z09DYkg4UHhNVXdPc1NzdVI4VTdDWTBVNE5qSFVWRmU2YUtSSDFSWTJRM0pZWTd6YVRnQTRfcF9lUTE0VHVqX0N4TjFYS0FTSGdfQmxkU0IyekVEdnJjaXlLb2FaMHpLb3pKclJFbkktX3MtTmtlRDdzRWVHYlHSAbMBQVVfeXFMT0lRTjhydFNjTllyUF9qalVtbW8zSVdvSUpJcS1fMlY0a3dFb2VhZWtzZXhXMzdXeXVYUHd5TzNBTDRWcmRHM0l2d21yVkdhZEVLWFA0cGJHWG5hYkNTOHpMNFRhZkpIcktLVnUwUExqSlN0X1BkOHQ4dk1oWGdFS01kOXlKVWxYWGdVMkRnNHlVV2IzWUJVVDE3LXRDWXF3NWViTm9OOXlWOGV6aFVEb0pHOWM?oc=5</t>
         </is>
       </c>
       <c r="F116" t="n">
         <v>7</v>
       </c>
       <c r="G116" s="1" t="n">
-        <v>46052.69449074074</v>
+        <v>46055.35223379629</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Fraud_Scam</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>The founder of First Brands, whose bankruptcy rattled Wall Street, charged in multibillion-dollar fraud - Business Insider</t>
+          <t>SPIE Photonics West 2026: AI Everywhere | Business | Jan 2026 - Photonics Spectra</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Thu, 29 Jan 2026 23:52:00 GMT</t>
+          <t>Mon, 02 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVk5Db3pJVzVlQ3c3bTdlaUswdUVFOHNET0I2Y3VfeGxpV011b0x2Zmdwa1JmQVJDdEpSNXBtaXR3NlF6SWc1eVY5dzcyQ1NKOW0yRFF4bEVkS20tcFVibW1sZUY0Q3VISUlQQVJZMEp6RzIwLUpHdkkySURkT3B5RXpyYkw3UW9hbjNRRWpiTFE3VEJvRlRNUFdNejZ5QTUwTHhlbA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOVER5ekZJMjhVaG1QdWFaMlNMU3R5QjY0U2RkY1JqQllOVDhOcUJQaHJOOEswMks5dmdRWHB0ZlNjV1dRa3BxRlZ0SVgyeXYxaTBQQmRpWEx1M1NfZlh2bmoxaUF3YzkyZnJXWlhDX2o0QlZ0bGdHY0NhNnlvRUZrWFJDR0hkaU5aRnBN?oc=5</t>
         </is>
       </c>
       <c r="F117" t="n">
         <v>7</v>
       </c>
       <c r="G117" s="1" t="n">
-        <v>46051.99444444444</v>
+        <v>46055.43611111111</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>How AI Is Changing the Storied McKinsey Interview - Business Insider</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 10:31:00 GMT</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPTGQyZlRzS3c2MDdEQ1JKaWIzYlFkOHZEY1JKZWx2bkRfRTBLQW9mTGM5ZWk2dmFXQnpVcHA2dEJ3QTBQRkVRQnVJMjhSejFKdTBXbHh3VGlRSGMtcEh1S0hhNnktem5VLWZFTEJGdUI5SXpDUTBHdEF3a0NoUVhSMXJyMk5ac1U?oc=5</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>7</v>
+      </c>
+      <c r="G118" s="1" t="n">
+        <v>46055.43819444445</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
           <t>Fraud_Scam</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Jersey businesses urged to beware of scam financial emails - BBC</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Tue, 27 Jan 2026 16:43:45 GMT</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1pWER4ajJRcUk3NHRXN0pMZkxGbWd4WjYzbnRzQUd2ZkwxNllfMXlFRElwSGpBSEJweHA1eXU0YnRlQldLcWFYdWU5NEFnNGNBcFF4X3RFOERzZ9IBX0FVX3lxTE1QckxlMlhjejd6enltLUl5ZzkyZ1VjeUlwcTJydUNqLUpGRVdVTTZXSkI0d1h0eUVNbS1KR3JHa3dVaVdyby0xWGVaWFJWVWwzRjFXYWwyMWxCTUlwSUxB?oc=5</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>7</v>
+      </c>
+      <c r="G119" s="1" t="n">
+        <v>46049.69704861111</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Email scams go QR - Insurance Business</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Fri, 30 Jan 2026 16:40:04 GMT</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQc2dSdFZPUVZpU29DWG42eFg3S21MdWZMNFdZY2p2cG1ha24tNmh1eWVkZk5Rc0tLYXN4SU1ORmg5WmRjbzQwaHJtMVVxM0gwb1FldUZScHJfXzVkbEp0bS02bkJERnRXMkhWOWxLcWEyYUhFUVJvQ0ZjSTY4MmRhbXVnODNMdmM?oc=5</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>7</v>
+      </c>
+      <c r="G120" s="1" t="n">
+        <v>46052.69449074074</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Scam emails claiming to be from Okotoks Oilers still circulating - OkotoksOnline</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 12:06:07 GMT</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNQ0txZE1iWXdHNlJjNVRKQ3g2SEN3YmJBdWNLTjd6RDJYbFMzYV9lYTJsZ1NUY1pCbmJ2REJ2YUxXQ1FtNXhCa3VCNDJfUmpGMGM4dnlaTTFvMnFXbF9VTlR0NzgxcWxYcGphclFISDFJZi1EVDUwd3BaWmY0NkY4V09wa0dzQ211TXpEV19uY1JSOWFxQlMxQjZ4SG41SjBY?oc=5</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>7</v>
+      </c>
+      <c r="G121" s="1" t="n">
+        <v>46055.50424768519</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>The founder of First Brands, whose bankruptcy rattled Wall Street, charged in multibillion-dollar fraud - Business Insider</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Thu, 29 Jan 2026 23:52:00 GMT</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVk5Db3pJVzVlQ3c3bTdlaUswdUVFOHNET0I2Y3VfeGxpV011b0x2Zmdwa1JmQVJDdEpSNXBtaXR3NlF6SWc1eVY5dzcyQ1NKOW0yRFF4bEVkS20tcFVibW1sZUY0Q3VISUlQQVJZMEp6RzIwLUpHdkkySURkT3B5RXpyYkw3UW9hbjNRRWpiTFE3VEJvRlRNUFdNejZ5QTUwTHhlbA?oc=5</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>7</v>
+      </c>
+      <c r="G122" s="1" t="n">
+        <v>46051.99444444444</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
         <is>
           <t>1st Circ. Upholds Atty's 7-Year Sentence In Email Fraud Case - Law360</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D123" t="inlineStr">
         <is>
           <t>Fri, 30 Jan 2026 21:32:00 GMT</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="E123" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxONDFkSVhyb0diX2ZlOWc2UlJjcjNtU2YxX3llS0ptSFBFV1ZScmt5Rkc2dHZoMHJ0TEFFYjc2cDZuc3dxV2N2N3k3S0tMT0NDVXc4R2FVcGUwZV9vUEpBS1FacUtTTlp6QnpuRGEwajROek9veWMzeWVjVUUyRXJoTWtMb3p1SEJRQ1JseG5ON3FGY21hdjZaZFp4SUxKdVZhWjJ0ZkYxQzNXS3RwNFdud3BB0gFeQVVfeXFMTmNOX0NRTVV2VEh3TFlCRjFjWXhoWWN6cUJnZzBuYVM1US1mR0tpb2ptNDFIcElrNC1WaVVZb05XSFc5TG5MVWRTRVhLMnRZcmFMc0tfS01WbFBlLTd1Zw?oc=5</t>
         </is>
       </c>
-      <c r="F118" t="n">
-        <v>7</v>
-      </c>
-      <c r="G118" s="1" t="n">
+      <c r="F123" t="n">
+        <v>7</v>
+      </c>
+      <c r="G123" s="1" t="n">
         <v>46052.89722222222</v>
       </c>
     </row>

</xml_diff>